<commit_message>
Add AI Audit Log - Week2
</commit_message>
<xml_diff>
--- a/AI Audit Log_HaMinhQuang.xlsx
+++ b/AI Audit Log_HaMinhQuang.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Assignment1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Assignment 2" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Assignment 3" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Assignment1" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Assignment2" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Assignment 3" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -36,6 +37,46 @@
     <t xml:space="preserve">Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
   </si>
   <si>
+    <t xml:space="preserve">Ví dụ: Abstraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI liệt kê 20 thuộc tính.
+Quyết định: Tôi chỉ chọn 10 thuộc tính liên quan đến chức năng đang được yêu cầu từ ứng dụng (CCCD, địa chỉ...) và lược bỏ 10 thuộc tính học thuật vì phù hợp với yêu cầu của ứng dụng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ví dụ: Process/Algorithm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI cung cấp code mẫu.
+Kiểm chứng: Tôi nhận thấy code AI chưa xử lý trường hợp mảng rỗng (Oversimplification). Tôi đã yêu cầu AI tối ưu lại và tự tay bổ sung điều kiện kiểm tra lỗi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ví dụ: Pattern Recognition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
+Kiểm chứng: AI đưa kết luận sai – không có giải thuật “tốt nhất” tuyệt đối (Hallucination). Mỗi giải thuật phù hợp với tình huống/context khác nhau.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ví dụ: Pattern Recognition + Literature Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
+Kiểm chứng: Tìm trên Google Scholar: 2/5 papers AI nêu là không tồn tại (fabrication). Tôi đã thay bằng 2 papers mà tôi đã tìm kiếm trên research gates và đã kiểm chứng trên google scholar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Abstraction</t>
   </si>
   <si>
@@ -88,6 +129,98 @@
   </si>
   <si>
     <t xml:space="preserve">Phản hồi: AI đưa ra các giai đoạn: Requirement → Design → Implementation → Testing → Deployment → Maintenance. Kiểm chứng: Tôi kiểm tra lại tài liệu môn học và thấy một số tài liệu tách riêng bước phân tích yêu cầu (Analysis), nên tôi chỉnh lại theo format giảng viên đã học để đồng nhất với slide môn học.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Xác định các class thực thể (entity classes) từ tập use case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Hệ thống IELTSPhobic của nhóm tôi có các use case về luyện thi, từ điển, diễn đàn và nâng cấp VIP. Theo Ch07 Static Modeling, làm sao tôi xác định được các entity class cần đưa vào class diagram? Có nên tạo class cho mọi danh từ xuất hiện trong SRS không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý dùng kỹ thuật "noun extraction" – gạch chân TẤT CẢ danh từ trong bản đặc tả rồi biến mỗi danh từ thành một class. AI liệt kê khoảng 40 class tiềm năng (Learner, Test, Question, Answer, Score, Forum, Post, Comment, Dictionary, Word, Plan, Payment, Email, Button, Page, Screen...).
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [OVERSIMPLIFICATION]: Gợi ý "mỗi danh từ một class" của AI quá máy móc. Nếu làm vậy sẽ sinh ra cả những class rác như Button, Page, Screen (thuộc tầng giao diện, không phải entity) và Email (thực ra là hành động/dịch vụ, không phải thực thể lưu trữ). Ch07 slide nhấn mạnh phải lọc danh từ theo tiêu chí: class entity là thứ có TRẠNG THÁI cần lưu trữ lâu dài và có ý nghĩa nghiệp vụ.
+• Contextualization: AI không biết rằng trong kiến trúc của nhóm, dữ liệu được lưu qua các bảng cụ thể (Learner, Test, Question, ForumPost, VipPlan, Transaction). Những thứ như Button/Page chỉ tồn tại ở tầng presentation nên không phải entity class.
+• Creative Synthesis: Tôi áp dụng noun extraction của AI làm bước SÀNG LỌC THÔ, rồi tự lọc lại theo 3 nhóm của Gomaa: entity class (lưu trạng thái – Learner, Test, Question, ForumPost, VipPlan, Transaction), boundary class (giao tiếp ngoài – StripeGateway, OpenAIService), control class (điều phối luồng – TestController, PaymentController). Loại bỏ Button/Page/Screen.
+• Decision Ownership: Tôi quyết định giữ lại 14 entity class cốt lõi, loại ~26 danh từ rác. Lý do: class diagram phải phản ánh đúng các bảng dữ liệu thật trong DB, nếu đưa cả class giao diện vào sẽ sai bản chất static model và mâu thuẫn với phần thiết kế CSDL ở Section IV.
+EVIDENCE: Bảng phân loại 14 entity / 2 boundary / 3 control class (Section III.1 báo cáo); đối chiếu schema DB thật.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Phân biệt Association, Aggregation và Composition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong class diagram, Test gồm nhiều Question, và Question thuộc về Test. Tôi nên dùng Aggregation hay Composition? Còn quan hệ giữa Learner và ForumPost thì là loại gì? Giải thích theo đúng định nghĩa UML."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Cả Test–Question lẫn Learner–ForumPost đều nên dùng Composition (hình thoi đặc), vì cái này chứa cái kia." AI giải thích Composition đơn giản là quan hệ "has-a" mạnh, dùng cho mọi trường hợp một đối tượng chứa đối tượng khác.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: Tôi nghi ngờ vì AI gộp hai trường hợp khác bản chất vào cùng một loại. Tra lại Ch07 (Class Relationships) và sách Gomaa: Composition (hình thoi đặc) hàm ý vòng đời PHỤ THUỘC – khi đối tượng chứa bị xóa thì đối tượng con cũng bị xóa theo, và con KHÔNG chia sẻ với cha khác. Aggregation (hình thoi rỗng) là quan hệ "whole-part" lỏng, con tồn tại độc lập. Phát hiện AI SAI: Learner–ForumPost không thể là Composition vì nếu xóa Learner, các bài forum thường vẫn được giữ lại (hiển thị "[deleted user]") – đó là Association/Aggregation, không phải Composition.
+• Contextualization: AI không biết business rule của nhóm: khi xóa tài khoản Learner, các ForumPost của họ vẫn được lưu để bảo toàn ngữ cảnh thảo luận. Còn Question thì thực sự bị xóa cùng Test (Question không tồn tại nếu không có Test).
+• Creative Synthesis: Tôi quyết định Test ◆— Question là Composition (đúng – vòng đời phụ thuộc, xóa Test thì Question đi theo), còn Learner —— ForumPost là Association một-nhiều bình thường (post sống độc lập với tài khoản). Bổ sung multiplicity rõ ràng: Test "1" — "1..*" Question; Learner "1" — "0..*" ForumPost.
+• Decision Ownership: Quyết định gắn đúng loại quan hệ + multiplicity cho từng cặp class. Lý do: chọn sai Composition/Aggregation sẽ kéo theo thiết kế ràng buộc khóa ngoại (cascade delete) sai trong DB – đây là lỗi bị trừ điểm nặng vì ảnh hưởng tới cả phần Implementation.
+CORRECTIVE ACTION: Sửa class diagram – đổi quan hệ Learner–ForumPost từ Composition (sai) sang Association; giữ Composition cho Test–Question.
+EVIDENCE: Class diagram trước/sau khi sửa (Figure III-1); đối chiếu Ch07 và ràng buộc ON DELETE trong schema.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Abstraction – Gán thuộc tính và kiểu dữ liệu cho class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Class VipPlan của tôi có các thuộc tính: id, tên gói, giá, thời hạn, ngày hết hạn của learner. Tôi nên đặt thuộc tính "ngày hết hạn VIP" ở class VipPlan hay class Learner? Nguyên tắc nào để quyết định một thuộc tính thuộc về class nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI giải thích đúng nguyên tắc cơ bản: một thuộc tính nên đặt ở class mà nó MÔ TẢ trực tiếp. AI gợi ý: giá/thời hạn mô tả gói nên thuộc VipPlan; còn "ngày hết hạn VIP của learner" mô tả trạng thái của từng learner cụ thể nên thuộc Learner, không thuộc VipPlan.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: Lần này AI ĐÚNG, khớp nguyên tắc Ch07: thuộc tính thuộc về class mà nó đặc trưng hóa. Tôi kiểm chứng bằng cách hỏi "giá trị này thay đổi theo gói hay theo người dùng?" – vipExpireAt thay đổi theo từng learner nên phải nằm ở Learner.
+• Contextualization: AI không biết chi tiết là hệ thống của tôi cho phép một Learner gia hạn nhiều lần và đổi gói, nên vipExpireAt là trạng thái động của Learner, còn lịch sử mua thì nằm ở class Transaction riêng. AI chỉ thấy mô tả tĩnh, không thấy luồng nghiệp vụ gia hạn.
+• Creative Synthesis: Tôi áp dụng nguyên tắc của AI nhưng tinh chỉnh theo mô hình thật: VipPlan giữ {planId, name, price, durationDays}; Learner giữ {..., vipExpireAt, isVip (derived)}; tách thêm Transaction {transId, learnerId, planId, amount, paidAt, status} để lưu lịch sử – chi tiết mà AI không gợi ý. Đánh dấu isVip là thuộc tính dẫn xuất (/isVip) tính từ vipExpireAt.
+• Decision Ownership: Quyết định phân bổ thuộc tính theo 3 class (VipPlan – Learner – Transaction) thay vì nhồi hết vào VipPlan như cách hiểu ban đầu. Lý do: tránh trùng lặp dữ liệu (data redundancy) và phản ánh đúng việc một learner có thể mua nhiều lần – phù hợp chuẩn hóa CSDL ở Section IV.
+EVIDENCE: Figure III-2 (cụm class VipPlan / Learner / Transaction) với multiplicity và thuộc tính dẫn xuất /isVip; đối chiếu bảng Transaction trong schema.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Ký hiệu visibility (+, -, #, ~) trong UML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong class diagram UML, các ký hiệu visibility +, -, # nghĩa là gì? Tôi đọc thấy có người dùng dấu ~. Dấu ~ có phải chuẩn UML không, và nó khác # thế nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI liệt kê: + là public, - là private, # là protected. Về dấu ~, AI nói "~ không phải ký hiệu UML chuẩn, có thể là ký hiệu tự chế của một số công cụ" và khuyên bỏ qua nó.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Sai do thiếu sót]: AI đúng 3 ký hiệu đầu nhưng SAI về dấu ~. Tôi tra lại tài liệu UML 2.x và sách Gomaa: dấu ~ LÀ ký hiệu UML chuẩn, biểu thị visibility "package" (đối tượng chỉ truy cập được trong cùng package/namespace). AI đã phủ nhận một ký hiệu hợp lệ và gắn nhãn "tự chế" cho nó.
+• Contextualization: Trong bối cảnh môn SWD392, mức package visibility (~) ít dùng nên dễ bị bỏ qua, nhưng nếu trong vấn đáp giảng viên hỏi mà mình trả lời "~ không chuẩn" theo AI thì sẽ bị coi là nắm sai chuẩn UML.
+• Creative Synthesis: Tôi xác nhận lại bằng UML spec 2.5.1 (mục Visibility) trước khi kết luận: có đủ 4 mức – public (+), private (-), protected (#), package (~). Quyết định trong class diagram của nhóm chủ yếu dùng - cho thuộc tính và + cho method (đóng gói chuẩn), không dùng ~ vì kiến trúc không chia package phức tạp – nhưng PHẢI biết ~ là chuẩn để không trả lời sai.
+• Decision Ownership: Quyết định phổ biến cho nhóm: thuộc tính để private (-), method public để (+); ghi chú lại rằng ~ (package) là hợp lệ dù nhóm không dùng. Lý do: vừa đảm bảo nguyên tắc encapsulation, vừa không hiểu sai chuẩn UML như AI gợi ý.
+CORRECTIVE ACTION: Rà soát class diagram – chuẩn hóa visibility: mọi attribute để -, mọi method public để +.
+EVIDENCE: UML spec 2.5.1 mục Visibility (4 mức gồm cả ~); Figure III-1 với visibility đã chuẩn hóa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Mô hình hóa kế thừa và class trừu tượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Hệ thống của tôi có 4 loại bài thi: Reading, Listening, Writing, Speaking. Chúng có thuộc tính chung (id, thời lượng, điểm) nhưng cách chấm khác nhau. Tôi nên mô hình hóa bằng generalization (kế thừa) thế nào? Có cần abstract class không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI đề xuất tạo 4 class Reading/Listening/Writing/Speaking hoàn toàn độc lập, mỗi class tự khai báo lại id, duration, score và method chấm điểm riêng. AI KHÔNG đề cập tới việc gom thuộc tính chung lên class cha hay dùng abstract class.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [OVERSIMPLIFICATION]: Cách của AI gây TRÙNG LẶP – 4 class lặp lại y hệt id, duration, score, vi phạm nguyên tắc tránh redundancy của Ch07/Ch08. Theo lý thuyết generalization, các thuộc tính/hành vi chung phải được "factor out" lên superclass.
+• Contextualization: AI không nắm được rằng cách chấm của Reading/Listening là tự động (so đáp án), còn Writing/Speaking cần AI feedback (chỉ VIP) – nghĩa là method gradeTest() có cùng chữ ký nhưng cài đặt khác nhau, đúng tình huống dùng polymorphism mà AI bỏ qua.
+• Creative Synthesis: Tôi thiết kế lại bằng generalization: tạo abstract class Test {id, duration, score; abstract gradeTest()} làm cha; 4 class con kế thừa và override gradeTest() theo cách riêng. Đánh dấu Test là abstract (in nghiêng tên class theo chuẩn UML) vì không bao giờ tạo instance "Test chung". Bổ sung ý: AutoGradedTest và AIGradedTest có thể là 2 lớp trung gian (Reading/Listening kế thừa AutoGradedTest; Writing/Speaking kế thừa AIGradedTest) để gom tiếp phần chung.
+• Decision Ownership: Quyết định dùng cây kế thừa 3 tầng (Test → AutoGradedTest/AIGradedTest → 4 skill) thay vì 4 class phẳng độc lập của AI. Lý do: thể hiện đúng quan hệ is-a, tận dụng polymorphism cho method gradeTest(), và phản ánh đúng business rule "AI feedback chỉ cho Writing/Speaking VIP" ngay trên class diagram.
+EVIDENCE: Figure III-3 (cây generalization Test) với abstract class in nghiêng và method gradeTest() được override; đối chiếu Ch07 phần Generalization/Specialization.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Phân tầng class theo stereotype (boundary / control / entity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi nghe nói class diagram nên chia theo 3 stereotype boundary, control, entity. Use case "Get AI feedback" gọi OpenAI thì OpenAIService là loại class nào? Còn class chứa logic gọi và xử lý kết quả thì sao? Giải thích theo Ch08."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời OpenAIService là boundary class (vì giao tiếp với hệ thống ngoài), và class xử lý logic là control class. AI giải thích entity = dữ liệu, boundary = giao diện/giao tiếp ngoài, control = điều phối – khớp mô hình BCE (Boundary-Control-Entity).
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG và khớp Ch08 (mô hình BCE/robustness analysis): boundary class là cầu nối giữa hệ thống và actor/hệ thống ngoài; control class điều phối luồng; entity class lưu trạng thái. Tôi kiểm chứng: boundary tiếp xúc "biên" hệ thống, đúng vai trò của một service gọi API ngoài.
+• Contextualization: AI không phân biệt một sắc thái: trong kiến trúc thật, OpenAIService của nhóm vừa làm nhiệm vụ boundary (gọi API) vừa chứa một ít logic ghép prompt – dễ bị lẫn vai trò. Đây là chi tiết kiến trúc mà định nghĩa lý thuyết không nói thẳng.
+• Creative Synthesis: Tôi quyết định TÁCH rõ trách nhiệm: OpenAIClient là boundary thuần (chỉ gửi/nhận HTTP với OpenAI), FeedbackController là control (nhận yêu cầu, kiểm tra quyền VIP, ghép prompt, gọi boundary, lưu kết quả), Feedback là entity (lưu nội dung feedback). Cách tách này giữ mỗi class một trách nhiệm (SRP) thay vì gộp vai trò như mô tả mơ hồ ban đầu.
+• Decision Ownership: Quyết định gán stereotype nhất quán toàn diagram: mọi class gọi hệ thống ngoài (OpenAIClient, StripeGateway, EmailSender) là «boundary»; mọi controller là «control»; mọi bảng dữ liệu là «entity». Lý do: tuân thủ mô hình BCE của Ch08, giúp diagram dễ ánh xạ sang kiến trúc phân tầng (layered architecture) ở Section II và sang sequence diagram ở Section III.
+EVIDENCE: Figure III-4 (class diagram phân tầng BCE cho luồng Get AI feedback) với 3 stereotype rõ ràng; đối chiếu Ch08 mô hình Boundary-Control-Entity.</t>
   </si>
 </sst>
 </file>
@@ -185,7 +318,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -204,6 +337,18 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -407,6 +552,102 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="45"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="71.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="71.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -435,84 +676,84 @@
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>6</v>
+      <c r="B2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>9</v>
+      <c r="B3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>12</v>
+      <c r="B4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>15</v>
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>18</v>
+      <c r="B6" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>21</v>
+      <c r="B7" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -526,25 +767,130 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="64.9"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="429.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="429.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="429.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="429.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="429.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="429.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>

</xml_diff>

<commit_message>
AI auditlog - Week3
</commit_message>
<xml_diff>
--- a/AI Audit Log_HaMinhQuang.xlsx
+++ b/AI Audit Log_HaMinhQuang.xlsx
@@ -5,13 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Assignment1" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Assignment2" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Assignment 3" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Assignment3" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -222,6 +222,46 @@
 • Decision Ownership: Quyết định gán stereotype nhất quán toàn diagram: mọi class gọi hệ thống ngoài (OpenAIClient, StripeGateway, EmailSender) là «boundary»; mọi controller là «control»; mọi bảng dữ liệu là «entity». Lý do: tuân thủ mô hình BCE của Ch08, giúp diagram dễ ánh xạ sang kiến trúc phân tầng (layered architecture) ở Section II và sang sequence diagram ở Section III.
 EVIDENCE: Figure III-4 (class diagram phân tầng BCE cho luồng Get AI feedback) với 3 stereotype rõ ràng; đối chiếu Ch08 mô hình Boundary-Control-Entity.</t>
   </si>
+  <si>
+    <t xml:space="preserve">Abstraction (Trừu tượng hóa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Liệt kê các lớp chính cần có trong một hệ thống quản lý học tập trực tuyến theo chuẩn Class Diagram."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI liệt kê: User, Course, Lesson, Quiz, Result.
+Quyết định: Thiếu phân biệt entity/control/boundary. Tôi bổ sung thêm lớp Enrollment và tách AuthService thành control class riêng.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decomposition (Phân rã vấn đề)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Hãy xác định các quan hệ giữa các lớp: User, Order, Product, Payment trong một hệ thống bán hàng."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI chỉ dùng Association cho tất cả các quan hệ.
+Kiểm chứng: Thiếu sót. Tôi phân tích lại: Order–Product là Aggregation, Order–Payment là Composition vì Payment không tồn tại nếu không có Order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pattern Recognition (Nhận dạng mẫu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong class diagram, khi nào nên dùng Inheritance thay vì Association để thể hiện quan hệ giữa hai lớp?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI khuyên dùng Inheritance khi hai lớp "có liên quan đến nhau".
+Kiểm chứng: Đây là Hallucination. Tôi xác nhận lại: chỉ dùng Inheritance khi thỏa mãn quan hệ "is-a", còn lại dùng Association.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Algorithm Design (Thiết kế thuật toán/Quy trình)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Xây dựng các bước để thiết kế Class Diagram từ đặc tả yêu cầu (SRS) cho một dự án phần mềm."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI đề xuất: đọc SRS → tìm danh từ → vẽ class → thêm method.
+Quyết định: Tôi bổ sung bước kiểm tra multiplicity và xác nhận quan hệ với team trước khi finalize diagram.</t>
+  </si>
 </sst>
 </file>
 
@@ -230,7 +270,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,6 +308,19 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -318,7 +371,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -361,6 +414,26 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -895,15 +968,92 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
AI audit log - Week 4
</commit_message>
<xml_diff>
--- a/AI Audit Log_HaMinhQuang.xlsx
+++ b/AI Audit Log_HaMinhQuang.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Assignment1" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Assignment2" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Assignment3" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Assignment4" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="82">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -261,6 +262,98 @@
   <si>
     <t xml:space="preserve">Phản hồi: AI đề xuất: đọc SRS → tìm danh từ → vẽ class → thêm method.
 Quyết định: Tôi bổ sung bước kiểm tra multiplicity và xác nhận quan hệ với team trước khi finalize diagram.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Decomposition – Phân tầng lifeline trong Sequence Diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi vẽ sequence diagram cho use case "Create Booking and Pay Deposit" của hệ thống AutoGo (đề Practical Exam). Đề bắt buộc dùng Repository Pattern và phải hiện rõ boundary, service/controller, repository, entity. Tôi nên đặt bao nhiêu lifeline và phân tầng thế nào cho đúng layered architecture?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý 4 lifeline: UI, BookingService, Repository, Booking entity. AI nói gộp Controller vào Service cho gọn vì "trong layered nhỏ thì controller và service có thể là một".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: Gợi ý gộp Controller vào Service là đơn giản hóa quá mức. Đề AutoGo yêu cầu RÕ RÀNG "a service OR controller component" và "repository components" (số nhiều). Nếu gộp thì mất đi tầng điều phối và chỉ có 1 repository, không thể hiện đúng Repository Pattern với nhiều repo (Car, Booking, Payment).
+• Contextualization: AI không biết Q1 (class diagram) của tôi đã tách rõ 5 tầng (Boundary-Control-Service-Repository-Domain). Đề nhấn mạnh "chosen architecture must be applied CONSISTENTLY throughout all diagrams" — nên sequence diagram phải khớp class diagram, không được gộp tầng tùy tiện.
+• Creative Synthesis: Tôi quyết định dùng đầy đủ các lifeline phân theo 5 tầng: BookingView (boundary), BookingController (control), BookingService + PaymentService (service), CarRepository + BookingRepository + PaymentRepository (repository), Booking + Payment (entity). Tách PaymentService riêng vì xử lý thanh toán là trách nhiệm khác (Single Responsibility).
+• Decision Ownership: Quyết định giữ đủ tầng + tách 3 repository riêng. Lý do: đảm bảo tính nhất quán với class diagram (Q1) và thể hiện Repository Pattern explicit như đề bắt buộc. Gộp tầng sẽ mất điểm "Repository Pattern usage must be explicit".
+EVIDENCE: Sequence diagram Q2 với 5 box phân tầng; đối chiếu class diagram Q1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Combined Fragment (alt / opt / loop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong sequence diagram, để mô hình hóa "nếu xe available thì tạo booking, nếu không thì báo lỗi" và "nếu thanh toán thành công thì confirm, thất bại thì cancel", tôi nên dùng combined fragment loại nào: alt, opt, hay break?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Dùng opt fragment cho cả hai trường hợp, vì opt thể hiện hành vi có điều kiện." AI nói opt linh hoạt hơn alt và dùng được cho mọi tình huống rẽ nhánh.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: AI SAI. Tôi tra lại định nghĩa UML combined fragment: OPT chỉ có MỘT nhánh (làm hoặc không làm — if không else); ALT có NHIỀU nhánh loại trừ nhau (if-else). Tình huống của tôi đều có 2 nhánh đối lập (available/NOT available; success/failed) → bắt buộc dùng ALT, không phải opt. Dùng opt sẽ không vẽ được nhánh "else" (báo lỗi / cancel booking).
+• Contextualization: Đề AutoGo ghi rõ "Conditional behavior must be modeled using ALT fragments for car availability and payment success or failure". Đề chỉ đích danh ALT, nên dùng opt là sai yêu cầu đề và mất điểm trực tiếp.
+• Creative Synthesis: Tôi dùng 2 alt fragment LỒNG NHAU: alt ngoài cho car availability (available / NOT available), alt trong cho payment (success / failed). Cách lồng này thể hiện đúng logic: chỉ thanh toán khi xe có sẵn.
+• Decision Ownership: Quyết định dùng alt (không phải opt) cho cả 2 nhánh, lồng nhau. Lý do: đúng định nghĩa UML (alt = nhiều nhánh loại trừ) và đúng yêu cầu tường minh của đề. Đây là lỗi dễ bị trừ điểm nếu nghe theo AI.
+CORRECTIVE ACTION: Dùng alt cho cả car-availability và payment, lồng alt payment trong nhánh "available".
+EVIDENCE: Sequence diagram Q2 với 2 alt fragment lồng nhau; đề Practical Exam Q2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Synchronous vs Asynchronous message &amp; return</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong sequence diagram IELTSPhobic use case "Upgrade to VIP", luồng thanh toán Stripe có phần webhook đến SAU khi user đã rời trang (bất đồng bộ). Tôi nên dùng loại mũi tên nào cho lời gọi đồng bộ và cho webhook bất đồng bộ? Return message vẽ thế nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI giải thích đúng: synchronous message dùng mũi tên đặc (filled arrowhead, -&gt;), asynchronous dùng mũi tên mở (open arrowhead, -&gt;&gt;), return message dùng nét đứt (--&gt;). AI gợi ý webhook Stripe nên là asynchronous message.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG về ký hiệu cơ bản (sync mũi tên đặc, async mũi tên mở, return nét đứt). Tôi kiểm chứng lại với chuẩn UML 2.x: đúng. Tuy nhiên AI chưa nói rõ cách thể hiện việc webhook đến ở một "thời điểm khác" trên cùng lifeline.
+• Contextualization: AI không biết kiến trúc thật: trong code repo, StripeWebhookController nhận event độc lập với luồng user bấm thanh toán (2 HTTP request riêng biệt, cách nhau về thời gian). Đây không chỉ là async message thường mà là 2 luồng tương tác tách biệt cần thể hiện rõ.
+• Creative Synthesis: Tôi quyết định tách sequence diagram VIP thành 2 phần rõ rệt: (1) Phase đồng bộ – user → controller → StripePaymentService → tạo checkout session (dùng sync message); (2) Phase bất đồng bộ – Stripe → StripeWebhookController → cập nhật VIP (dùng async message -&gt;&gt; ở đầu vào). Thêm ghi chú "asynchronous webhook" để người đọc hiểu khoảng cách thời gian.
+• Decision Ownership: Quyết định dùng sync cho luồng nội bộ, async (-&gt;&gt;)  cho webhook Stripe đến, return nét đứt cho mọi phản hồi. Lý do: phản ánh đúng bản chất bất đồng bộ của thanh toán và khớp với code StripeWebhookController thật.
+EVIDENCE: Sequence diagram UC-09 (2 phase sync/async); StripeWebhookController.cs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Abstraction – Ký hiệu chuẩn của Sequence Diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Sequence diagram theo chuẩn UML có những thành phần nào bắt buộc? Tôi nghe nói có ký hiệu "self-loop arrow" và "found message". Activation bar (thanh kích hoạt) có bắt buộc không? Object trong sequence có cần gạch chân tên không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời sequence diagram bắt buộc có: lifeline, message, activation bar, và "tên object PHẢI gạch chân giống object diagram". AI khẳng định gạch chân tên object là quy tắc bắt buộc trong mọi sequence diagram UML.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Fabrication/Context Misunderstanding]: AI SAI ở điểm "tên object bắt buộc gạch chân". Tôi tra lại chuẩn UML 2.x và tài liệu môn học: việc gạch chân (underline) tên là quy ước của INSTANCE trong object diagram, KHÔNG bắt buộc trong sequence diagram. Trong sequence diagram, lifeline thường ghi dạng "objectName : ClassName" và đa số công cụ (PlantUML, Visual Paradigm) KHÔNG gạch chân. AI trộn lẫn quy ước object diagram vào sequence diagram.
+• Contextualization: Trong bối cảnh dùng PlantUML để vẽ (công cụ tôi đang dùng), không có cú pháp bắt buộc gạch chân lifeline. Nếu cố làm theo AI sẽ tốn công vô ích và không đúng thực hành phổ biến.
+• Creative Synthesis: Tôi xác minh bằng 2 nguồn (chuẩn UML + tài liệu Gomaa) trước khi kết luận. Giữ đúng các thành phần thật sự cần: lifeline (participant), message (sync/async/return), activation bar (activate/deactivate), và combined fragment (alt). Bỏ qua yêu cầu "gạch chân" sai của AI.
+• Decision Ownership: Quyết định KHÔNG gạch chân tên lifeline; dùng format "name : Class" theo chuẩn phổ biến. Activation bar thì CÓ dùng (activate/deactivate) vì nó thể hiện rõ thời gian một object đang xử lý — hữu ích dù không tuyệt đối bắt buộc. Lý do: tuân thủ chuẩn UML đúng cho sequence diagram, tránh áp nhầm quy ước của diagram khác.
+CORRECTIVE ACTION: Dùng lifeline không gạch chân; giữ activation bar để thể hiện control focus.
+EVIDENCE: Chuẩn UML 2.x Interaction diagrams; sequence diagram đã vẽ bằng PlantUML.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Ánh xạ message trong Sequence sang method code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi muốn sequence diagram cho use case "Add Listening Test" của IELTSPhobic khớp đúng với code thật. Trong code có ExamController, ExamService, ExamRepository, CloudinaryService. Thứ tự gọi method và tên message nên đặt thế nào cho đúng code?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI đề xuất luồng chung: View → Controller.Create → Service.Create → Repository.Add → SaveChanges. AI đặt tên message generic như "save()", "create()", "store()".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: Luồng tổng thể AI đúng (đúng thứ tự tầng), nhưng tên message generic ("save", "store") KHÔNG khớp method thật trong code. Sequence diagram tốt phải dùng đúng tên method thật để traceable.
+• Contextualization: AI không đọc được code repo nên không biết tên method chính xác. Tôi mở các file thật: ExamController có Create(CreateExamDto), ExamService có Create(dto), ExamRepository có Add(exam) + SaveChanges(), và phần upload audio gọi CloudinaryService.UploadAudio() trả về URL. Đây là chi tiết chỉ có khi đọc code.
+• Creative Synthesis: Tôi viết lại sequence diagram dùng ĐÚNG tên method từ code: AdminTestView -&gt; ExamController : Create(CreateExamDto); ExamController -&gt; CloudinaryService : UploadAudio(file); ExamController -&gt; ExamService : Create(dto); ExamService -&gt; ExamRepository : Add(exam); ExamRepository -&gt; DbContext : SaveChanges(). Thêm cả nhánh trả về URL từ Cloudinary trước khi save.
+• Decision Ownership: Quyết định đặt tên message khớp 1-1 với method trong code thật, không dùng tên generic. Lý do: đảm bảo traceability giữa sequence diagram (Section III) và code (Section V) — khi vấn đáp giảng viên có thể đối chiếu trực tiếp với GitHub.
+EVIDENCE: Sequence diagram UC-57; ExamController.cs, ExamService.cs, ExamRepostiory.cs, CloudinaryService.cs trong repo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Mức độ chi tiết: Analysis vs Design level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Khi vẽ sequence diagram cho báo cáo SWD392, tôi nên vẽ ở mức analysis (chỉ boundary-control-entity theo MVC) hay design (đủ controller-service-repository-entity khớp code)? Hai mức này khác nhau ra sao và nên chọn mức nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI giải thích analysis-level sequence dùng stereotype boundary/control/entity (theo phân tích MVC), còn design-level thêm các class thật như service, repository. AI khuyên "dùng design-level cho mọi trường hợp vì chi tiết hơn".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI giải thích đúng sự khác biệt 2 mức, nhưng lời khuyên "luôn dùng design-level" hơi cứng nhắc. Tùy mục đích từng phần báo cáo mà chọn mức phù hợp — analysis-level giúp hiểu nghiệp vụ, design-level giúp map sang code.
+• Contextualization: Báo cáo SWD392 của nhóm có cả Section II (Analysis) và Section III-IV (Design). Giảng viên trước đó đã nhận xét class diagram của nhóm "mới ở mức entity, chưa hoàn chỉnh" — nên với phần design, phải dùng design-level đủ tầng (service + repository) mới đạt. Đây là bối cảnh quan trọng AI không biết.
+• Creative Synthesis: Tôi quyết định dùng 2 mức cho 2 phần khác nhau: (1) Section II Analysis Models → sequence analysis-level (boundary-control-entity) để thể hiện luồng nghiệp vụ; (2) Section III/IV Design → sequence design-level đầy đủ (controller-service-repository-entity) khớp Repository Pattern trong code. Hai mức bổ trợ nhau, không mâu thuẫn.
+• Decision Ownership: Quyết định phân biệt rõ analysis-level cho phần phân tích và design-level cho phần thiết kế. Lý do: đáp ứng nhận xét của giảng viên (cần đủ tầng ở phần design) đồng thời giữ phần analysis gọn để dễ hiểu nghiệp vụ. Thể hiện hiểu biết về vai trò khác nhau của 2 mức thay vì áp dụng máy móc 1 mức.
+EVIDENCE: Sequence analysis-level (Section II) + design-level (Section III); nhận xét của giảng viên về class diagram.</t>
   </si>
 </sst>
 </file>
@@ -371,7 +464,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -416,24 +509,32 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -971,10 +1072,10 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -991,7 +1092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
@@ -1045,6 +1146,129 @@
       </c>
       <c r="D5" s="15" t="s">
         <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="69.7"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="449.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AI audit log - Week 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_HaMinhQuang.xlsx
+++ b/AI Audit Log_HaMinhQuang.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,6 +13,7 @@
     <sheet name="Assignment2" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Assignment3" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Assignment4" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Assignment5" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="100">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -354,6 +355,98 @@
 • Creative Synthesis: Tôi quyết định dùng 2 mức cho 2 phần khác nhau: (1) Section II Analysis Models → sequence analysis-level (boundary-control-entity) để thể hiện luồng nghiệp vụ; (2) Section III/IV Design → sequence design-level đầy đủ (controller-service-repository-entity) khớp Repository Pattern trong code. Hai mức bổ trợ nhau, không mâu thuẫn.
 • Decision Ownership: Quyết định phân biệt rõ analysis-level cho phần phân tích và design-level cho phần thiết kế. Lý do: đáp ứng nhận xét của giảng viên (cần đủ tầng ở phần design) đồng thời giữ phần analysis gọn để dễ hiểu nghiệp vụ. Thể hiện hiểu biết về vai trò khác nhau của 2 mức thay vì áp dụng máy móc 1 mức.
 EVIDENCE: Sequence analysis-level (Section II) + design-level (Section III); nhận xét của giảng viên về class diagram.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Xác định state-dependent object cần vẽ State Diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Hệ thống IELTSPhobic có 26 entity. Theo Ch10 (Finite State Machines &amp; Statecharts), không phải object nào cũng cần state diagram. Tôi nên vẽ state diagram cho những object nào? Tiêu chí để xác định một object là state-dependent là gì?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý vẽ state diagram cho TẤT CẢ entity chính: User, Exam, ExamAttempt, Post, Comment, Payment, VocabGroup... AI nói "vẽ càng nhiều càng đầy đủ, thể hiện được nhiều trạng thái".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: Gợi ý "vẽ cho tất cả" của AI là sai. Theo Ch10, chỉ object STATE-DEPENDENT mới cần state diagram — tức object có hành vi PHỤ THUỘC vào trạng thái hiện tại và đi qua nhiều trạng thái rõ rệt theo thời gian. Những object như Word, Tag, VocabGroup chỉ là dữ liệu tĩnh (CRUD thuần), không có state machine ý nghĩa → vẽ state diagram cho chúng là thừa và sai khái niệm.
+• Contextualization: AI không biết bản chất nghiệp vụ từng entity. Trong IELTSPhobic, chỉ vài object thực sự đổi trạng thái theo vòng đời: ExamAttempt (NotStarted → InProgress → Submitted → Scored), Post (Pending → Published → Hidden), User VIP status (NonVIP → VIP → hết hạn). Word/Tag thì không có "vòng đời trạng thái".
+• Creative Synthesis: Tôi lập tiêu chí lọc dựa trên Ch10: object được chọn phải (1) có ≥3 trạng thái phân biệt, (2) hành vi khác nhau tùy trạng thái, (3) có event làm chuyển trạng thái. Áp tiêu chí này, tôi chọn 3 object: ExamAttempt, Post, User (VIP status). Loại các entity dữ liệu tĩnh.
+• Decision Ownership: Quyết định chỉ vẽ state diagram cho 3 state-dependent object thay vì cả 26. Lý do: đúng khái niệm Ch10 (statechart chỉ cho state-dependent object), tránh vẽ thừa làm loãng báo cáo. Đây cũng là cách case study FOS làm — chỉ vẽ state cho News object.
+EVIDENCE: 3 state diagram (ExamAttempt, Post, User VIP); Ch10 định nghĩa state-dependent object.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Phân biệt State và Activity/Action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Cho state diagram của Order (đề Practical Exam Vincom): các state nên đặt tên là gì? Tôi định đặt: Creating, Confirming, Paying, Cooking, Serving. Đặt như vậy đúng chưa?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng rồi, các tên Creating, Confirming, Paying, Cooking, Serving thể hiện rõ hệ thống đang làm gì ở mỗi giai đoạn." AI xác nhận cách đặt tên động từ-ing này là chuẩn cho state.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: AI SAI. Tôi tra lại Ch10: STATE là một TRẠNG THÁI (danh từ/tính từ, mô tả object ĐANG Ở ĐÂU), không phải HÀNH ĐỘNG đang diễn ra. "Cooking", "Paying" là activity/action (động từ tiến hành), thuộc về activity diagram. State đúng phải là danh từ chỉ tình trạng đã đạt: Created, Confirmed, Paid, Preparing, Served... AI nhầm lẫn state với activity.
+• Contextualization: Đề Vincom ghi rõ các state cần có: Created, Confirmed, Paid, Preparing, ReadyToServe, Served, Completed — toàn bộ là danh từ/quá khứ phân từ chỉ trạng thái, KHÔNG phải động từ-ing. Nếu đặt "Paying" thay vì "Paid" sẽ sai yêu cầu đề và sai khái niệm state.
+• Creative Synthesis: Tôi sửa toàn bộ tên state về dạng trạng thái: Created (đã tạo), Confirmed (đã xác nhận), Paid (đã trả tiền), Preparing (đang ở trạng thái được chuẩn bị — đây là ngoại lệ chấp nhận được vì mô tả tình trạng kéo dài), ReadyToServe (sẵn sàng phục vụ), Served (đã phục vụ), Completed (hoàn tất). Event mới là động từ (confirmOrder, paySuccess) đặt trên transition.
+• Decision Ownership: Quyết định state = danh từ/trạng thái, event = động từ trên mũi tên. Lý do: đúng định nghĩa Ch10 và khớp tên state đề yêu cầu. Đây là lỗi cơ bản rất hay bị trừ điểm vì nhầm state diagram thành activity diagram.
+CORRECTIVE ACTION: Đổi Creating→Created, Paying→Paid, Cooking→Preparing, Serving→Served. Động từ chỉ dùng cho event.
+EVIDENCE: Ch10 (state là trạng thái, không phải action); đề Vincom Q3 liệt kê tên state chuẩn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Cú pháp transition: event [guard] / action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong state diagram User VIP của IELTSPhobic, từ trạng thái Paid muốn chuyển sang VIP nhưng chỉ khi webhook Stripe xác thực thành công, và đồng thời phải cập nhật VipExpireAt. Tôi viết transition này thế nào cho đúng cú pháp UML?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời đúng cú pháp: transition viết dạng "event [guard condition] / action". Cụ thể: webhookReceived [signatureValid] / updateVipExpireAt. AI giải thích event kích hoạt, guard là điều kiện phải đúng, action là việc làm khi chuyển.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG, khớp Ch10. Tôi kiểm chứng cú pháp: event là bắt buộc, [guard] và /action là tùy chọn. Transition chỉ kích hoạt khi event xảy ra VÀ guard đúng.
+• Contextualization: AI không biết chi tiết kỹ thuật: trong code IELTSPhobic, việc kích hoạt VIP do StripeWebhookController xử lý sau khi verify signature. Nên guard condition [signatureValid] phản ánh đúng business rule BR "VIP chỉ kích hoạt khi webhook hợp lệ" — chi tiết mà chỉ người đọc code mới biết.
+• Creative Synthesis: Tôi viết các transition của state diagram User VIP với đầy đủ guard + action: NonVIP --&gt; VIP : paySuccess [signatureValid] / setVipExpireAt; VIP --&gt; NonVIP : expire [now &gt; VipExpireAt]; VIP --&gt; VIP : renew [paySuccess] / extendVipExpireAt (self-transition gia hạn). Thêm self-transition mà AI không gợi ý.
+• Decision Ownership: Quyết định dùng đầy đủ cú pháp event [guard] / action cho các transition quan trọng, đặc biệt thêm guard [signatureValid] để phản ánh bảo mật webhook. Lý do: thể hiện chính xác điều kiện chuyển trạng thái và khớp logic code thật, không chỉ vẽ mũi tên trống.
+EVIDENCE: State diagram User VIP với guard/action; StripeWebhookController.cs; Ch10 cú pháp transition.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Abstraction – Composite state &amp; thành phần bắt buộc của Statechart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"State diagram theo chuẩn UML bắt buộc phải có những thành phần nào? Tôi nghe nói mọi state diagram đều phải dùng composite state (nested state) và phải có history state (H). Có đúng không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng, state diagram chuẩn UML BẮT BUỘC phải có composite state để nhóm các trạng thái, và phải có history state (H) để nhớ trạng thái trước đó." AI khẳng định đây là yêu cầu bắt buộc của mọi statechart.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Fabrication/Logic Error]: AI SAI. Tôi tra lại Ch10: thành phần BẮT BUỘC của state diagram chỉ gồm: initial state, các state, transition (với event), và final state. Composite state (state lồng nhau) và history state (H) là tính năng NÂNG CAO, chỉ dùng KHI CẦN cho hệ thống phức tạp, hoàn toàn KHÔNG bắt buộc. Phần lớn state diagram đơn giản (như Order lifecycle, ExamAttempt) không cần composite/history state. AI bịa ra yêu cầu bắt buộc không tồn tại.
+• Contextualization: Trong bối cảnh đề Practical Exam Vincom, yêu cầu chỉ là: initial + final state, ≥6 states, ≥6 transitions có event, ≥1 nhánh rẽ. KHÔNG hề yêu cầu composite hay history state. Nếu cố thêm vào theo lời AI sẽ làm diagram phức tạp vô ích và lệch yêu cầu đề.
+• Creative Synthesis: Tôi xác minh bằng đề thi + Ch10, kết luận chỉ dùng các thành phần cơ bản. Giữ state diagram Order phẳng (flat) với 9 state + transition rõ ràng, KHÔNG dùng composite/history. Chỉ cân nhắc composite state nếu sau này có nhóm trạng thái con thực sự (vd nhóm "InKitchen" gồm Preparing + ReadyToServe) — nhưng không bắt buộc.
+• Decision Ownership: Quyết định dùng state diagram phẳng với thành phần cơ bản, KHÔNG ép composite/history state. Lý do: đúng yêu cầu đề và đúng Ch10 (các tính năng nâng cao chỉ dùng khi cần). Tránh làm rối diagram để "trông phức tạp" một cách giả tạo.
+CORRECTIVE ACTION: Giữ state diagram phẳng, bỏ ý định thêm composite/history state.
+EVIDENCE: Ch10 (composite/history là optional); đề Vincom Q3 (không yêu cầu composite).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Mô hình hóa nhánh rẽ và final state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"State diagram Order của tôi có luồng chính Created → Confirmed → Paid → Preparing → Served → Completed. Nhưng cần xử lý trường hợp thanh toán thất bại và hủy đơn. Tôi nên mô hình các nhánh thất bại này thế nào? Có cần final state riêng cho mỗi nhánh không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý thêm 1 state PaymentFailed cho thanh toán thất bại và dẫn về cùng 1 final state với luồng thành công. AI nói "tất cả nên về chung 1 final state cho gọn".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng phần "thêm state PaymentFailed" nhưng phần "tất cả về chung 1 final state" là chưa chính xác về mặt ngữ nghĩa. Theo Ch10, một state diagram có thể có NHIỀU final state để biểu thị các cách kết thúc khác nhau. Gộp tất cả về 1 final state vẫn hợp lệ về cú pháp, nhưng tách ra rõ ràng hơn cho người đọc hiểu các kịch bản kết thúc.
+• Contextualization: Đề Vincom yêu cầu "alternative termination state such as Cancelled or PaymentFailed" và "at least one branching path". Nghĩa là cần thể hiện RÕ các nhánh thất bại như những trạng thái kết thúc riêng, không gộp mờ vào happy path.
+• Creative Synthesis: Tôi thiết kế 2 nhánh rẽ riêng: (1) Confirmed --&gt; PaymentFailed : payFail; (2) Created/Confirmed --&gt; Cancelled : cancelOrder. Cả PaymentFailed và Cancelled đều dẫn về final state [*]. Happy path Served --&gt; Completed --&gt; [*]. Như vậy có 3 đường tới final state, thể hiện rõ 3 kịch bản kết thúc (thành công, thanh toán lỗi, bị hủy).
+• Decision Ownership: Quyết định tách rõ 2 nhánh thất bại (PaymentFailed, Cancelled) như các trạng thái kết thúc riêng trước khi về final state. Lý do: đáp ứng yêu cầu đề "alternative termination + branching path", và giúp người đọc thấy rõ mọi kịch bản kết thúc của Order.
+EVIDENCE: State diagram Order với 3 nhánh kết thúc; đề Vincom Q3 yêu cầu alternative termination.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Pattern Recognition – Tính nhất quán giữa State Diagram và các model khác</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"State diagram của News/Post object có event DisableNews, EnableNews. Các event này có cần trùng tên với message trong sequence diagram và use case không? Hay đặt tên tự do cũng được?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nói "Tên event trong state diagram đặt tự do miễn dễ hiểu, không nhất thiết trùng với sequence diagram vì chúng là các diagram độc lập."
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Context Misunderstanding]: AI hiểu sai. Theo nguyên tắc mô hình hóa nhất quán (và như case study FOS minh họa rõ): các event gây chuyển trạng thái trong state diagram NÊN trùng tên với các message tương ứng đến state-dependent object trong sequence/communication diagram. Đây không phải bắt buộc cú pháp nhưng là best practice để đảm bảo traceability giữa các model.
+• Contextualization: Case study FOS (tài liệu RDS môn học) ghi rõ: "The events DisableNews and EnableNews cause state transitions to share the same names as two messages arriving at the state-dependent object in the sequence diagrams". Đây là chuẩn mực mà giảng viên dạy theo — AI không biết bối cảnh tài liệu môn học này.
+• Creative Synthesis: Tôi quyết định đồng bộ tên event xuyên suốt 3 model: trong sequence diagram có message DisableNews() gửi đến News object → trong state diagram News có transition Enable --&gt; Disable : DisableNews → trong use case có UC Disable News. Ba cái dùng chung 1 tên, tạo traceability.
+• Decision Ownership: Quyết định đặt tên event state diagram TRÙNG với message sequence diagram và tên use case. Lý do: đảm bảo tính nhất quán giữa các model (yêu cầu quan trọng khi chấm điểm), giúp người đọc và giảng viên truy vết từ use case → sequence → state. Không đặt tên tùy tiện như AI gợi ý.
+EVIDENCE: State diagram News/Post; sequence diagram Disable/Enable News; case study FOS (RDS) về tính nhất quán event-message.</t>
   </si>
 </sst>
 </file>
@@ -464,7 +557,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -527,6 +620,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1167,108 +1264,231 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="69.7"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="449.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="419.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="69.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="71.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="n">
+      <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="n">
+      <c r="B2" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>69</v>
+      <c r="B3" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="449.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="n">
+      <c r="B4" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="434.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>75</v>
+      <c r="B5" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="n">
+      <c r="B6" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>81</v>
+      <c r="B7" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AI audit log - Week 6
</commit_message>
<xml_diff>
--- a/AI Audit Log_HaMinhQuang.xlsx
+++ b/AI Audit Log_HaMinhQuang.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Assignment2" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Assignment3" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Assignment4" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Assignment5" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Assignment6" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Assignment5" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="118">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -355,6 +356,98 @@
 • Creative Synthesis: Tôi quyết định dùng 2 mức cho 2 phần khác nhau: (1) Section II Analysis Models → sequence analysis-level (boundary-control-entity) để thể hiện luồng nghiệp vụ; (2) Section III/IV Design → sequence design-level đầy đủ (controller-service-repository-entity) khớp Repository Pattern trong code. Hai mức bổ trợ nhau, không mâu thuẫn.
 • Decision Ownership: Quyết định phân biệt rõ analysis-level cho phần phân tích và design-level cho phần thiết kế. Lý do: đáp ứng nhận xét của giảng viên (cần đủ tầng ở phần design) đồng thời giữ phần analysis gọn để dễ hiểu nghiệp vụ. Thể hiện hiểu biết về vai trò khác nhau của 2 mức thay vì áp dụng máy móc 1 mức.
 EVIDENCE: Sequence analysis-level (Section II) + design-level (Section III); nhận xét của giảng viên về class diagram.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Chọn đúng loại diagram: Activity vs Sequence vs State</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi đã có sequence diagram và state diagram cho use case "Upgrade to VIP" của IELTSPhobic. Giờ có cần vẽ thêm activity diagram cho cùng use case này không? Activity diagram khác sequence và state diagram ở điểm gì, và khi nào nên dùng nó?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nói activity diagram, sequence diagram và state diagram là "giống nhau, đều mô tả luồng xử lý", nên "có thể chọn 1 trong 3 tùy thích, không cần vẽ cả ba". AI gợi ý bỏ activity diagram vì đã có sequence.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI sai khi coi 3 diagram là "giống nhau, thay thế được". Thực ra mỗi cái mô hình một khía cạnh khác: Activity diagram mô tả LUỒNG CÔNG VIỆC/workflow (các bước hoạt động và rẽ nhánh, có thể song song); Sequence diagram mô tả TƯƠNG TÁC giữa các object theo thời gian (ai gọi ai); State diagram mô tả VÒNG ĐỜI TRẠNG THÁI của 1 object. Chúng bổ trợ nhau, không thay thế.
+• Contextualization: AI không biết yêu cầu báo cáo SWD392 + case study FOS dùng activity diagram để mô hình hóa event flow của use case (Manage Product, Add Product) ở phần Requirement, còn sequence/state ở phần Analysis. Mỗi diagram phục vụ một phase khác nhau trong tài liệu.
+• Creative Synthesis: Tôi quyết định dùng activity diagram cho phần REQUIREMENT (II.5.3) để mô tả luồng nghiệp vụ của use case một cách dễ hiểu cho stakeholder; dùng sequence diagram cho phần ANALYSIS (III) để thể hiện tương tác object; dùng state diagram cho object có vòng đời. Ba cái cùng tồn tại, mỗi cái một mục đích.
+• Decision Ownership: Quyết định GIỮ activity diagram cho phần requirement, không bỏ như AI khuyên. Lý do: activity diagram dễ đọc cho người không chuyên kỹ thuật và là cầu nối giữa use case description (văn xuôi) với sequence diagram (kỹ thuật). Đúng cách case study FOS làm.
+EVIDENCE: Activity diagram phần II.5.3; sequence ở III; case study FOS dùng cả 3 loại.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Phân biệt Decision Node và Fork/Join</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong activity diagram UC-11 Start Practice Listening, hệ thống vừa auto-save mỗi 5 giây VỪA cho học viên trả lời câu hỏi (2 việc diễn ra đồng thời). Còn chỗ kiểm tra "câu trả lời hợp lệ hay không" thì rẽ 2 hướng. Cả hai chỗ này dùng ký hiệu hình thoi decision node phải không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng, cả hai đều dùng hình thoi (diamond) decision node. Decision node xử lý được cả rẽ nhánh điều kiện lẫn việc song song." AI khẳng định diamond dùng cho mọi trường hợp phân nhánh.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: AI SAI. Tôi tra lại lý thuyết activity diagram: DECISION NODE (hình thoi ◇) dùng cho rẽ nhánh ĐIỀU KIỆN — chọn 1 trong nhiều đường tùy guard (if-else). Còn FORK/JOIN (thanh đậm ▬) dùng cho luồng SONG SONG — tách thành nhiều luồng chạy đồng thời rồi gộp lại. Hai ký hiệu hoàn toàn khác nhau. Auto-save chạy SONG SONG với trả lời câu hỏi → phải dùng FORK, không phải decision node.
+• Contextualization: AI không hiểu bản chất kỹ thuật: trong code IELTSPhobic, auto-save (mỗi 5s) và việc học viên nhập đáp án là 2 tiến trình độc lập chạy đồng thời (concurrent), không phải rẽ nhánh chọn một. Đây là chi tiết từ thiết kế thực tế.
+• Creative Synthesis: Tôi tách rõ 2 ký hiệu trong activity diagram: (1) FORK (thanh đậm) tách luồng "trả lời câu hỏi" và luồng "auto-save mỗi 5s" chạy song song, sau đó JOIN lại khi submit; (2) DECISION node (hình thoi) cho chỗ "đáp án hợp lệ? / timer hết giờ?" rẽ nhánh điều kiện. Dùng đúng ký hiệu cho đúng ngữ cảnh.
+• Decision Ownership: Quyết định dùng FORK/JOIN cho hành vi song song và DECISION node cho rẽ nhánh điều kiện, KHÔNG gộp chung như AI nói. Lý do: đúng ngữ nghĩa UML activity diagram và phản ánh đúng hành vi concurrent của hệ thống. Dùng sai ký hiệu sẽ bị trừ điểm và hiểu sai luồng.
+CORRECTIVE ACTION: Auto-save dùng FORK (song song); validation dùng DECISION node.
+EVIDENCE: Activity diagram UC-11 với fork (auto-save) + decision (validate); lý thuyết activity diagram (decision vs fork).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Decomposition – Swimlane (Partition) phân chia trách nhiệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Activity diagram UC-09 Upgrade to VIP có 4 bên tham gia: Learner, System, Stripe Gateway, Email Service. Làm sao thể hiện rõ mỗi hoạt động thuộc về bên nào? Có cần swimlane không và chia thế nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI giải thích đúng khái niệm swimlane (partition): chia activity diagram thành các làn dọc/ngang, mỗi làn ứng với một actor/component, đặt hoạt động vào làn của bên chịu trách nhiệm. AI gợi ý 4 swimlane cho 4 bên.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG về khái niệm swimlane. Tôi kiểm chứng: swimlane giúp thể hiện rõ AI/bên nào thực hiện hoạt động nào — tăng tính rõ ràng về trách nhiệm. Mỗi action nằm trong đúng làn của chủ thể thực hiện.
+• Contextualization: AI không biết chi tiết luồng VIP có phần bất đồng bộ: webhook từ Stripe đến SAU khi Learner đã rời trang. Nên swimlane Stripe Gateway và System có tương tác ở 2 thời điểm khác nhau (lúc tạo checkout và lúc nhận webhook) — cần thể hiện cẩn thận trong cùng diagram.
+• Creative Synthesis: Tôi thiết kế 4 swimlane (Learner | System | Stripe Gateway | Email Service) và sắp xếp hoạt động theo 2 giai đoạn: giai đoạn đồng bộ (Learner chọn plan → System tạo checkout → Stripe hiện form → Learner trả tiền) và giai đoạn bất đồng bộ (Stripe gửi webhook → System verify + cập nhật VIP → Email gửi xác nhận). Mỗi action đặt đúng làn chủ thể.
+• Decision Ownership: Quyết định dùng 4 swimlane phản ánh đúng 4 bên tham gia, sắp xếp hoạt động theo trình tự đồng bộ rồi bất đồng bộ. Lý do: thể hiện rõ trách nhiệm từng bên và làm nổi bật phần webhook bất đồng bộ — đặc trưng kỹ thuật quan trọng của luồng thanh toán.
+EVIDENCE: Activity diagram UC-09 với 4 swimlane; StripeWebhookController.cs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Abstraction – Activity Diagram (UML) vs Flowchart truyền thống</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Activity diagram có phải chỉ là flowchart (lưu đồ thuật toán) vẽ lại không? Tôi có thể dùng activity diagram để mô tả chi tiết từng dòng code if/else/for trong method GradeWriting() được không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng, activity diagram chính là flowchart, dùng để mô tả chi tiết logic code từng dòng if/else/for trong một method. Bạn nên vẽ activity diagram cho mọi method phức tạp để thể hiện thuật toán."
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Context Misunderstanding/Oversimplification]: AI nhầm lẫn. Activity diagram (UML) và flowchart truyền thống KHÁC nhau về mục đích: flowchart mô tả thuật toán mức code (chi tiết từng lệnh); activity diagram UML mô tả LUỒNG NGHIỆP VỤ / workflow ở mức cao hơn (các bước hoạt động, ai làm, rẽ nhánh nghiệp vụ, song song), và có thêm khái niệm swimlane, fork/join mà flowchart không có. Vẽ activity diagram để mô tả từng dòng if/else trong code là sai mục đích — đó là lạm dụng, làm diagram vụn vặt và sai tầm trừu tượng.
+• Contextualization: Trong báo cáo SWD392, activity diagram dùng để mô hình hóa event flow của USE CASE (mức nghiệp vụ), không phải mô tả implementation chi tiết method GradeWriting(). Code chi tiết để ở Section V (code snippet), không vẽ activity cho nó.
+• Creative Synthesis: Tôi giữ activity diagram ở mức use case event flow: ví dụ UC-26 Get Writing AI Feedback chỉ mô tả các bước "submit bài → gửi tới AI → nhận điểm → hiển thị feedback", KHÔNG đi sâu vào vòng lặp parse JSON hay xử lý lỗi chi tiết của code. Giữ đúng tầm trừu tượng nghiệp vụ.
+• Decision Ownership: Quyết định dùng activity diagram ở mức workflow nghiệp vụ của use case, KHÔNG vẽ cho từng method code. Lý do: đúng mục đích activity diagram trong UML/COMET, giữ tầm trừu tượng phù hợp với tài liệu thiết kế, tránh lạm dụng thành flowchart code vụn vặt.
+CORRECTIVE ACTION: Activity diagram chỉ ở mức use case event flow, không mô tả chi tiết code method.
+EVIDENCE: Activity diagram UC mức nghiệp vụ; phân biệt activity diagram UML vs flowchart.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Mô hình hóa main flow, alternative flow và exception</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Activity diagram UC-01 Register có luồng chính (nhập thông tin → tạo tài khoản → gửi OTP → xác thực) và các nhánh phụ (dữ liệu không hợp lệ, OTP sai). Làm sao thể hiện main flow, alternative flow và exception trong cùng 1 activity diagram?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý dùng initial node (chấm đặc) bắt đầu, các action node cho từng bước, decision node cho chỗ kiểm tra (valid? OTP đúng?), và final node kết thúc. AI gợi ý nhánh lỗi quay lại bước nhập liệu (loop).
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng cấu trúc cơ bản (initial → actions → decision → final). Tôi kiểm chứng khớp với cách case study FOS vẽ activity diagram Add Product (có decision "is data valid?" và "is system error?"). Tuy nhiên AI chưa nói rõ cách thể hiện exception (E6.1, E7.1) tách biệt với alternative flow.
+• Contextualization: AI không biết use case description UC-01 của tôi đã định nghĩa rõ: Alternative flow (ALT-1: chọn đăng ký Google thay vì email) và Exception (EXC-1: dữ liệu sai, EXC-2: OTP sai). Activity diagram cần phản ánh đúng các nhánh này khớp với use case description.
+• Creative Synthesis: Tôi thiết kế activity diagram UC-01 với: main flow đi thẳng; decision "dữ liệu hợp lệ?" → nhánh No quay lại form (exception EXC-1); decision "OTP đúng?" → nhánh No cho resend tối đa 3 lần (exception EXC-2); main flow kết thúc ở final node "account verified". Mỗi decision tương ứng đúng 1 exception trong use case description.
+• Decision Ownership: Quyết định để activity diagram khớp 1-1 với use case description (main/alt/exception). Lý do: đảm bảo traceability giữa use case description (văn xuôi) và activity diagram (đồ họa) — khi vấn đáp có thể đối chiếu trực tiếp, và đúng vai trò activity diagram là mô hình hóa event flow của use case.
+EVIDENCE: Activity diagram UC-01 khớp use case description; case study FOS activity Add Product.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Pattern Recognition – Chọn use case nào để vẽ activity diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Hệ thống IELTSPhobic có 72 use case. Tôi có cần vẽ activity diagram cho TẤT CẢ 72 use case không? Nếu không thì chọn vẽ cho những use case nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI khuyên "vẽ activity diagram cho tất cả use case để báo cáo đầy đủ và chuyên nghiệp". AI nói càng nhiều diagram càng được đánh giá cao.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI sai về số lượng. Vẽ 72 activity diagram là không cần thiết và phản tác dụng — nhiều use case đơn giản (như "View forum posts", "Logout") chỉ có 1-2 bước tuyến tính, không có rẽ nhánh, vẽ activity diagram là thừa. Case study FOS chỉ vẽ activity cho 2 use case tiêu biểu (Manage Product, Add Product) có luồng đủ phức tạp.
+• Contextualization: AI không biết tiêu chí chọn của môn học: chỉ vẽ activity diagram cho use case có event flow ĐỦ PHỨC TẠP (có alternative flow, exception, hoặc nhánh song song). Use case CRUD đơn giản không cần.
+• Creative Synthesis: Tôi lập tiêu chí chọn use case để vẽ activity: (1) có nhiều bước, (2) có rẽ nhánh điều kiện hoặc song song, (3) có alternative/exception flow. Áp tiêu chí, tôi chọn 6 use case tiêu biểu cùng bộ với phần mô tả chi tiết: UC-01 Register, UC-04 Login, UC-09 Upgrade VIP, UC-11 Start Practice, UC-55 Suspend User, UC-57 Add Listening Test. Bỏ các UC CRUD đơn giản.
+• Decision Ownership: Quyết định chỉ vẽ activity diagram cho 6 use case phức tạp tiêu biểu, không vẽ cả 72. Lý do: tập trung vào use case có giá trị mô hình hóa cao, tránh báo cáo loãng với hàng chục diagram tầm thường. Chất lượng hơn số lượng — đúng cách case study FOS làm.
+EVIDENCE: 6 activity diagram tiêu biểu (II.5.3); case study FOS chỉ vẽ 2 activity.</t>
   </si>
   <si>
     <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Xác định state-dependent object cần vẽ State Diagram</t>
@@ -1390,7 +1483,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="71.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="69.8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1407,7 +1500,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
@@ -1435,7 +1528,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="344.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="n">
         <v>3</v>
       </c>
@@ -1449,7 +1542,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="434.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="449.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
@@ -1463,7 +1556,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
@@ -1477,7 +1570,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="344.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
@@ -1489,6 +1582,129 @@
       </c>
       <c r="D7" s="18" t="s">
         <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="71.7"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="464.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AI Audit log - Week 7
</commit_message>
<xml_diff>
--- a/AI Audit Log_HaMinhQuang.xlsx
+++ b/AI Audit Log_HaMinhQuang.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,8 +13,9 @@
     <sheet name="Assignment2" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Assignment3" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Assignment4" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Assignment6" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Assignment5" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Assignment5" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Assignment6" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Assignment7" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="136">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -358,6 +359,98 @@
 EVIDENCE: Sequence analysis-level (Section II) + design-level (Section III); nhận xét của giảng viên về class diagram.</t>
   </si>
   <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Xác định state-dependent object cần vẽ State Diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Hệ thống IELTSPhobic có 26 entity. Theo Ch10 (Finite State Machines &amp; Statecharts), không phải object nào cũng cần state diagram. Tôi nên vẽ state diagram cho những object nào? Tiêu chí để xác định một object là state-dependent là gì?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý vẽ state diagram cho TẤT CẢ entity chính: User, Exam, ExamAttempt, Post, Comment, Payment, VocabGroup... AI nói "vẽ càng nhiều càng đầy đủ, thể hiện được nhiều trạng thái".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: Gợi ý "vẽ cho tất cả" của AI là sai. Theo Ch10, chỉ object STATE-DEPENDENT mới cần state diagram — tức object có hành vi PHỤ THUỘC vào trạng thái hiện tại và đi qua nhiều trạng thái rõ rệt theo thời gian. Những object như Word, Tag, VocabGroup chỉ là dữ liệu tĩnh (CRUD thuần), không có state machine ý nghĩa → vẽ state diagram cho chúng là thừa và sai khái niệm.
+• Contextualization: AI không biết bản chất nghiệp vụ từng entity. Trong IELTSPhobic, chỉ vài object thực sự đổi trạng thái theo vòng đời: ExamAttempt (NotStarted → InProgress → Submitted → Scored), Post (Pending → Published → Hidden), User VIP status (NonVIP → VIP → hết hạn). Word/Tag thì không có "vòng đời trạng thái".
+• Creative Synthesis: Tôi lập tiêu chí lọc dựa trên Ch10: object được chọn phải (1) có ≥3 trạng thái phân biệt, (2) hành vi khác nhau tùy trạng thái, (3) có event làm chuyển trạng thái. Áp tiêu chí này, tôi chọn 3 object: ExamAttempt, Post, User (VIP status). Loại các entity dữ liệu tĩnh.
+• Decision Ownership: Quyết định chỉ vẽ state diagram cho 3 state-dependent object thay vì cả 26. Lý do: đúng khái niệm Ch10 (statechart chỉ cho state-dependent object), tránh vẽ thừa làm loãng báo cáo. Đây cũng là cách case study FOS làm — chỉ vẽ state cho News object.
+EVIDENCE: 3 state diagram (ExamAttempt, Post, User VIP); Ch10 định nghĩa state-dependent object.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Phân biệt State và Activity/Action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Cho state diagram của Order (đề Practical Exam Vincom): các state nên đặt tên là gì? Tôi định đặt: Creating, Confirming, Paying, Cooking, Serving. Đặt như vậy đúng chưa?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng rồi, các tên Creating, Confirming, Paying, Cooking, Serving thể hiện rõ hệ thống đang làm gì ở mỗi giai đoạn." AI xác nhận cách đặt tên động từ-ing này là chuẩn cho state.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error]: AI SAI. Tôi tra lại Ch10: STATE là một TRẠNG THÁI (danh từ/tính từ, mô tả object ĐANG Ở ĐÂU), không phải HÀNH ĐỘNG đang diễn ra. "Cooking", "Paying" là activity/action (động từ tiến hành), thuộc về activity diagram. State đúng phải là danh từ chỉ tình trạng đã đạt: Created, Confirmed, Paid, Preparing, Served... AI nhầm lẫn state với activity.
+• Contextualization: Đề Vincom ghi rõ các state cần có: Created, Confirmed, Paid, Preparing, ReadyToServe, Served, Completed — toàn bộ là danh từ/quá khứ phân từ chỉ trạng thái, KHÔNG phải động từ-ing. Nếu đặt "Paying" thay vì "Paid" sẽ sai yêu cầu đề và sai khái niệm state.
+• Creative Synthesis: Tôi sửa toàn bộ tên state về dạng trạng thái: Created (đã tạo), Confirmed (đã xác nhận), Paid (đã trả tiền), Preparing (đang ở trạng thái được chuẩn bị — đây là ngoại lệ chấp nhận được vì mô tả tình trạng kéo dài), ReadyToServe (sẵn sàng phục vụ), Served (đã phục vụ), Completed (hoàn tất). Event mới là động từ (confirmOrder, paySuccess) đặt trên transition.
+• Decision Ownership: Quyết định state = danh từ/trạng thái, event = động từ trên mũi tên. Lý do: đúng định nghĩa Ch10 và khớp tên state đề yêu cầu. Đây là lỗi cơ bản rất hay bị trừ điểm vì nhầm state diagram thành activity diagram.
+CORRECTIVE ACTION: Đổi Creating→Created, Paying→Paid, Cooking→Preparing, Serving→Served. Động từ chỉ dùng cho event.
+EVIDENCE: Ch10 (state là trạng thái, không phải action); đề Vincom Q3 liệt kê tên state chuẩn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Cú pháp transition: event [guard] / action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong state diagram User VIP của IELTSPhobic, từ trạng thái Paid muốn chuyển sang VIP nhưng chỉ khi webhook Stripe xác thực thành công, và đồng thời phải cập nhật VipExpireAt. Tôi viết transition này thế nào cho đúng cú pháp UML?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời đúng cú pháp: transition viết dạng "event [guard condition] / action". Cụ thể: webhookReceived [signatureValid] / updateVipExpireAt. AI giải thích event kích hoạt, guard là điều kiện phải đúng, action là việc làm khi chuyển.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG, khớp Ch10. Tôi kiểm chứng cú pháp: event là bắt buộc, [guard] và /action là tùy chọn. Transition chỉ kích hoạt khi event xảy ra VÀ guard đúng.
+• Contextualization: AI không biết chi tiết kỹ thuật: trong code IELTSPhobic, việc kích hoạt VIP do StripeWebhookController xử lý sau khi verify signature. Nên guard condition [signatureValid] phản ánh đúng business rule BR "VIP chỉ kích hoạt khi webhook hợp lệ" — chi tiết mà chỉ người đọc code mới biết.
+• Creative Synthesis: Tôi viết các transition của state diagram User VIP với đầy đủ guard + action: NonVIP --&gt; VIP : paySuccess [signatureValid] / setVipExpireAt; VIP --&gt; NonVIP : expire [now &gt; VipExpireAt]; VIP --&gt; VIP : renew [paySuccess] / extendVipExpireAt (self-transition gia hạn). Thêm self-transition mà AI không gợi ý.
+• Decision Ownership: Quyết định dùng đầy đủ cú pháp event [guard] / action cho các transition quan trọng, đặc biệt thêm guard [signatureValid] để phản ánh bảo mật webhook. Lý do: thể hiện chính xác điều kiện chuyển trạng thái và khớp logic code thật, không chỉ vẽ mũi tên trống.
+EVIDENCE: State diagram User VIP với guard/action; StripeWebhookController.cs; Ch10 cú pháp transition.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Abstraction – Composite state &amp; thành phần bắt buộc của Statechart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"State diagram theo chuẩn UML bắt buộc phải có những thành phần nào? Tôi nghe nói mọi state diagram đều phải dùng composite state (nested state) và phải có history state (H). Có đúng không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng, state diagram chuẩn UML BẮT BUỘC phải có composite state để nhóm các trạng thái, và phải có history state (H) để nhớ trạng thái trước đó." AI khẳng định đây là yêu cầu bắt buộc của mọi statechart.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Fabrication/Logic Error]: AI SAI. Tôi tra lại Ch10: thành phần BẮT BUỘC của state diagram chỉ gồm: initial state, các state, transition (với event), và final state. Composite state (state lồng nhau) và history state (H) là tính năng NÂNG CAO, chỉ dùng KHI CẦN cho hệ thống phức tạp, hoàn toàn KHÔNG bắt buộc. Phần lớn state diagram đơn giản (như Order lifecycle, ExamAttempt) không cần composite/history state. AI bịa ra yêu cầu bắt buộc không tồn tại.
+• Contextualization: Trong bối cảnh đề Practical Exam Vincom, yêu cầu chỉ là: initial + final state, ≥6 states, ≥6 transitions có event, ≥1 nhánh rẽ. KHÔNG hề yêu cầu composite hay history state. Nếu cố thêm vào theo lời AI sẽ làm diagram phức tạp vô ích và lệch yêu cầu đề.
+• Creative Synthesis: Tôi xác minh bằng đề thi + Ch10, kết luận chỉ dùng các thành phần cơ bản. Giữ state diagram Order phẳng (flat) với 9 state + transition rõ ràng, KHÔNG dùng composite/history. Chỉ cân nhắc composite state nếu sau này có nhóm trạng thái con thực sự (vd nhóm "InKitchen" gồm Preparing + ReadyToServe) — nhưng không bắt buộc.
+• Decision Ownership: Quyết định dùng state diagram phẳng với thành phần cơ bản, KHÔNG ép composite/history state. Lý do: đúng yêu cầu đề và đúng Ch10 (các tính năng nâng cao chỉ dùng khi cần). Tránh làm rối diagram để "trông phức tạp" một cách giả tạo.
+CORRECTIVE ACTION: Giữ state diagram phẳng, bỏ ý định thêm composite/history state.
+EVIDENCE: Ch10 (composite/history là optional); đề Vincom Q3 (không yêu cầu composite).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Mô hình hóa nhánh rẽ và final state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"State diagram Order của tôi có luồng chính Created → Confirmed → Paid → Preparing → Served → Completed. Nhưng cần xử lý trường hợp thanh toán thất bại và hủy đơn. Tôi nên mô hình các nhánh thất bại này thế nào? Có cần final state riêng cho mỗi nhánh không?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý thêm 1 state PaymentFailed cho thanh toán thất bại và dẫn về cùng 1 final state với luồng thành công. AI nói "tất cả nên về chung 1 final state cho gọn".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI đúng phần "thêm state PaymentFailed" nhưng phần "tất cả về chung 1 final state" là chưa chính xác về mặt ngữ nghĩa. Theo Ch10, một state diagram có thể có NHIỀU final state để biểu thị các cách kết thúc khác nhau. Gộp tất cả về 1 final state vẫn hợp lệ về cú pháp, nhưng tách ra rõ ràng hơn cho người đọc hiểu các kịch bản kết thúc.
+• Contextualization: Đề Vincom yêu cầu "alternative termination state such as Cancelled or PaymentFailed" và "at least one branching path". Nghĩa là cần thể hiện RÕ các nhánh thất bại như những trạng thái kết thúc riêng, không gộp mờ vào happy path.
+• Creative Synthesis: Tôi thiết kế 2 nhánh rẽ riêng: (1) Confirmed --&gt; PaymentFailed : payFail; (2) Created/Confirmed --&gt; Cancelled : cancelOrder. Cả PaymentFailed và Cancelled đều dẫn về final state [*]. Happy path Served --&gt; Completed --&gt; [*]. Như vậy có 3 đường tới final state, thể hiện rõ 3 kịch bản kết thúc (thành công, thanh toán lỗi, bị hủy).
+• Decision Ownership: Quyết định tách rõ 2 nhánh thất bại (PaymentFailed, Cancelled) như các trạng thái kết thúc riêng trước khi về final state. Lý do: đáp ứng yêu cầu đề "alternative termination + branching path", và giúp người đọc thấy rõ mọi kịch bản kết thúc của Order.
+EVIDENCE: State diagram Order với 3 nhánh kết thúc; đề Vincom Q3 yêu cầu alternative termination.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Pattern Recognition – Tính nhất quán giữa State Diagram và các model khác</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"State diagram của News/Post object có event DisableNews, EnableNews. Các event này có cần trùng tên với message trong sequence diagram và use case không? Hay đặt tên tự do cũng được?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nói "Tên event trong state diagram đặt tự do miễn dễ hiểu, không nhất thiết trùng với sequence diagram vì chúng là các diagram độc lập."
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Context Misunderstanding]: AI hiểu sai. Theo nguyên tắc mô hình hóa nhất quán (và như case study FOS minh họa rõ): các event gây chuyển trạng thái trong state diagram NÊN trùng tên với các message tương ứng đến state-dependent object trong sequence/communication diagram. Đây không phải bắt buộc cú pháp nhưng là best practice để đảm bảo traceability giữa các model.
+• Contextualization: Case study FOS (tài liệu RDS môn học) ghi rõ: "The events DisableNews and EnableNews cause state transitions to share the same names as two messages arriving at the state-dependent object in the sequence diagrams". Đây là chuẩn mực mà giảng viên dạy theo — AI không biết bối cảnh tài liệu môn học này.
+• Creative Synthesis: Tôi quyết định đồng bộ tên event xuyên suốt 3 model: trong sequence diagram có message DisableNews() gửi đến News object → trong state diagram News có transition Enable --&gt; Disable : DisableNews → trong use case có UC Disable News. Ba cái dùng chung 1 tên, tạo traceability.
+• Decision Ownership: Quyết định đặt tên event state diagram TRÙNG với message sequence diagram và tên use case. Lý do: đảm bảo tính nhất quán giữa các model (yêu cầu quan trọng khi chấm điểm), giúp người đọc và giảng viên truy vết từ use case → sequence → state. Không đặt tên tùy tiện như AI gợi ý.
+EVIDENCE: State diagram News/Post; sequence diagram Disable/Enable News; case study FOS (RDS) về tính nhất quán event-message.</t>
+  </si>
+  <si>
     <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Chọn đúng loại diagram: Activity vs Sequence vs State</t>
   </si>
   <si>
@@ -450,96 +543,96 @@
 EVIDENCE: 6 activity diagram tiêu biểu (II.5.3); case study FOS chỉ vẽ 2 activity.</t>
   </si>
   <si>
-    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Xác định state-dependent object cần vẽ State Diagram</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Hệ thống IELTSPhobic có 26 entity. Theo Ch10 (Finite State Machines &amp; Statecharts), không phải object nào cũng cần state diagram. Tôi nên vẽ state diagram cho những object nào? Tiêu chí để xác định một object là state-dependent là gì?"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý vẽ state diagram cho TẤT CẢ entity chính: User, Exam, ExamAttempt, Post, Comment, Payment, VocabGroup... AI nói "vẽ càng nhiều càng đầy đủ, thể hiện được nhiều trạng thái".
-HUMAN DELTA &amp; REFLECTION:
-• Critical Thinking [Oversimplification]: Gợi ý "vẽ cho tất cả" của AI là sai. Theo Ch10, chỉ object STATE-DEPENDENT mới cần state diagram — tức object có hành vi PHỤ THUỘC vào trạng thái hiện tại và đi qua nhiều trạng thái rõ rệt theo thời gian. Những object như Word, Tag, VocabGroup chỉ là dữ liệu tĩnh (CRUD thuần), không có state machine ý nghĩa → vẽ state diagram cho chúng là thừa và sai khái niệm.
-• Contextualization: AI không biết bản chất nghiệp vụ từng entity. Trong IELTSPhobic, chỉ vài object thực sự đổi trạng thái theo vòng đời: ExamAttempt (NotStarted → InProgress → Submitted → Scored), Post (Pending → Published → Hidden), User VIP status (NonVIP → VIP → hết hạn). Word/Tag thì không có "vòng đời trạng thái".
-• Creative Synthesis: Tôi lập tiêu chí lọc dựa trên Ch10: object được chọn phải (1) có ≥3 trạng thái phân biệt, (2) hành vi khác nhau tùy trạng thái, (3) có event làm chuyển trạng thái. Áp tiêu chí này, tôi chọn 3 object: ExamAttempt, Post, User (VIP status). Loại các entity dữ liệu tĩnh.
-• Decision Ownership: Quyết định chỉ vẽ state diagram cho 3 state-dependent object thay vì cả 26. Lý do: đúng khái niệm Ch10 (statechart chỉ cho state-dependent object), tránh vẽ thừa làm loãng báo cáo. Đây cũng là cách case study FOS làm — chỉ vẽ state cho News object.
-EVIDENCE: 3 state diagram (ExamAttempt, Post, User VIP); Ch10 định nghĩa state-dependent object.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Phân biệt State và Activity/Action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Cho state diagram của Order (đề Practical Exam Vincom): các state nên đặt tên là gì? Tôi định đặt: Creating, Confirming, Paying, Cooking, Serving. Đặt như vậy đúng chưa?"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng rồi, các tên Creating, Confirming, Paying, Cooking, Serving thể hiện rõ hệ thống đang làm gì ở mỗi giai đoạn." AI xác nhận cách đặt tên động từ-ing này là chuẩn cho state.
-HUMAN DELTA &amp; REFLECTION:
-• Critical Thinking [HALLUCINATION – Logic Error]: AI SAI. Tôi tra lại Ch10: STATE là một TRẠNG THÁI (danh từ/tính từ, mô tả object ĐANG Ở ĐÂU), không phải HÀNH ĐỘNG đang diễn ra. "Cooking", "Paying" là activity/action (động từ tiến hành), thuộc về activity diagram. State đúng phải là danh từ chỉ tình trạng đã đạt: Created, Confirmed, Paid, Preparing, Served... AI nhầm lẫn state với activity.
-• Contextualization: Đề Vincom ghi rõ các state cần có: Created, Confirmed, Paid, Preparing, ReadyToServe, Served, Completed — toàn bộ là danh từ/quá khứ phân từ chỉ trạng thái, KHÔNG phải động từ-ing. Nếu đặt "Paying" thay vì "Paid" sẽ sai yêu cầu đề và sai khái niệm state.
-• Creative Synthesis: Tôi sửa toàn bộ tên state về dạng trạng thái: Created (đã tạo), Confirmed (đã xác nhận), Paid (đã trả tiền), Preparing (đang ở trạng thái được chuẩn bị — đây là ngoại lệ chấp nhận được vì mô tả tình trạng kéo dài), ReadyToServe (sẵn sàng phục vụ), Served (đã phục vụ), Completed (hoàn tất). Event mới là động từ (confirmOrder, paySuccess) đặt trên transition.
-• Decision Ownership: Quyết định state = danh từ/trạng thái, event = động từ trên mũi tên. Lý do: đúng định nghĩa Ch10 và khớp tên state đề yêu cầu. Đây là lỗi cơ bản rất hay bị trừ điểm vì nhầm state diagram thành activity diagram.
-CORRECTIVE ACTION: Đổi Creating→Created, Paying→Paid, Cooking→Preparing, Serving→Served. Động từ chỉ dùng cho event.
-EVIDENCE: Ch10 (state là trạng thái, không phải action); đề Vincom Q3 liệt kê tên state chuẩn.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Cú pháp transition: event [guard] / action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Trong state diagram User VIP của IELTSPhobic, từ trạng thái Paid muốn chuyển sang VIP nhưng chỉ khi webhook Stripe xác thực thành công, và đồng thời phải cập nhật VipExpireAt. Tôi viết transition này thế nào cho đúng cú pháp UML?"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời đúng cú pháp: transition viết dạng "event [guard condition] / action". Cụ thể: webhookReceived [signatureValid] / updateVipExpireAt. AI giải thích event kích hoạt, guard là điều kiện phải đúng, action là việc làm khi chuyển.
-HUMAN DELTA &amp; REFLECTION:
-• Critical Thinking: AI ĐÚNG, khớp Ch10. Tôi kiểm chứng cú pháp: event là bắt buộc, [guard] và /action là tùy chọn. Transition chỉ kích hoạt khi event xảy ra VÀ guard đúng.
-• Contextualization: AI không biết chi tiết kỹ thuật: trong code IELTSPhobic, việc kích hoạt VIP do StripeWebhookController xử lý sau khi verify signature. Nên guard condition [signatureValid] phản ánh đúng business rule BR "VIP chỉ kích hoạt khi webhook hợp lệ" — chi tiết mà chỉ người đọc code mới biết.
-• Creative Synthesis: Tôi viết các transition của state diagram User VIP với đầy đủ guard + action: NonVIP --&gt; VIP : paySuccess [signatureValid] / setVipExpireAt; VIP --&gt; NonVIP : expire [now &gt; VipExpireAt]; VIP --&gt; VIP : renew [paySuccess] / extendVipExpireAt (self-transition gia hạn). Thêm self-transition mà AI không gợi ý.
-• Decision Ownership: Quyết định dùng đầy đủ cú pháp event [guard] / action cho các transition quan trọng, đặc biệt thêm guard [signatureValid] để phản ánh bảo mật webhook. Lý do: thể hiện chính xác điều kiện chuyển trạng thái và khớp logic code thật, không chỉ vẽ mũi tên trống.
-EVIDENCE: State diagram User VIP với guard/action; StripeWebhookController.cs; Ch10 cú pháp transition.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERIFICATION | DTC: Abstraction – Composite state &amp; thành phần bắt buộc của Statechart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"State diagram theo chuẩn UML bắt buộc phải có những thành phần nào? Tôi nghe nói mọi state diagram đều phải dùng composite state (nested state) và phải có history state (H). Có đúng không?"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng, state diagram chuẩn UML BẮT BUỘC phải có composite state để nhóm các trạng thái, và phải có history state (H) để nhớ trạng thái trước đó." AI khẳng định đây là yêu cầu bắt buộc của mọi statechart.
-HUMAN DELTA &amp; REFLECTION:
-• Critical Thinking [HALLUCINATION – Fabrication/Logic Error]: AI SAI. Tôi tra lại Ch10: thành phần BẮT BUỘC của state diagram chỉ gồm: initial state, các state, transition (với event), và final state. Composite state (state lồng nhau) và history state (H) là tính năng NÂNG CAO, chỉ dùng KHI CẦN cho hệ thống phức tạp, hoàn toàn KHÔNG bắt buộc. Phần lớn state diagram đơn giản (như Order lifecycle, ExamAttempt) không cần composite/history state. AI bịa ra yêu cầu bắt buộc không tồn tại.
-• Contextualization: Trong bối cảnh đề Practical Exam Vincom, yêu cầu chỉ là: initial + final state, ≥6 states, ≥6 transitions có event, ≥1 nhánh rẽ. KHÔNG hề yêu cầu composite hay history state. Nếu cố thêm vào theo lời AI sẽ làm diagram phức tạp vô ích và lệch yêu cầu đề.
-• Creative Synthesis: Tôi xác minh bằng đề thi + Ch10, kết luận chỉ dùng các thành phần cơ bản. Giữ state diagram Order phẳng (flat) với 9 state + transition rõ ràng, KHÔNG dùng composite/history. Chỉ cân nhắc composite state nếu sau này có nhóm trạng thái con thực sự (vd nhóm "InKitchen" gồm Preparing + ReadyToServe) — nhưng không bắt buộc.
-• Decision Ownership: Quyết định dùng state diagram phẳng với thành phần cơ bản, KHÔNG ép composite/history state. Lý do: đúng yêu cầu đề và đúng Ch10 (các tính năng nâng cao chỉ dùng khi cần). Tránh làm rối diagram để "trông phức tạp" một cách giả tạo.
-CORRECTIVE ACTION: Giữ state diagram phẳng, bỏ ý định thêm composite/history state.
-EVIDENCE: Ch10 (composite/history là optional); đề Vincom Q3 (không yêu cầu composite).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Algorithms – Mô hình hóa nhánh rẽ và final state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"State diagram Order của tôi có luồng chính Created → Confirmed → Paid → Preparing → Served → Completed. Nhưng cần xử lý trường hợp thanh toán thất bại và hủy đơn. Tôi nên mô hình các nhánh thất bại này thế nào? Có cần final state riêng cho mỗi nhánh không?"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI RESPONSE (Summary): AI gợi ý thêm 1 state PaymentFailed cho thanh toán thất bại và dẫn về cùng 1 final state với luồng thành công. AI nói "tất cả nên về chung 1 final state cho gọn".
-HUMAN DELTA &amp; REFLECTION:
-• Critical Thinking: AI đúng phần "thêm state PaymentFailed" nhưng phần "tất cả về chung 1 final state" là chưa chính xác về mặt ngữ nghĩa. Theo Ch10, một state diagram có thể có NHIỀU final state để biểu thị các cách kết thúc khác nhau. Gộp tất cả về 1 final state vẫn hợp lệ về cú pháp, nhưng tách ra rõ ràng hơn cho người đọc hiểu các kịch bản kết thúc.
-• Contextualization: Đề Vincom yêu cầu "alternative termination state such as Cancelled or PaymentFailed" và "at least one branching path". Nghĩa là cần thể hiện RÕ các nhánh thất bại như những trạng thái kết thúc riêng, không gộp mờ vào happy path.
-• Creative Synthesis: Tôi thiết kế 2 nhánh rẽ riêng: (1) Confirmed --&gt; PaymentFailed : payFail; (2) Created/Confirmed --&gt; Cancelled : cancelOrder. Cả PaymentFailed và Cancelled đều dẫn về final state [*]. Happy path Served --&gt; Completed --&gt; [*]. Như vậy có 3 đường tới final state, thể hiện rõ 3 kịch bản kết thúc (thành công, thanh toán lỗi, bị hủy).
-• Decision Ownership: Quyết định tách rõ 2 nhánh thất bại (PaymentFailed, Cancelled) như các trạng thái kết thúc riêng trước khi về final state. Lý do: đáp ứng yêu cầu đề "alternative termination + branching path", và giúp người đọc thấy rõ mọi kịch bản kết thúc của Order.
-EVIDENCE: State diagram Order với 3 nhánh kết thúc; đề Vincom Q3 yêu cầu alternative termination.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DECISION-MAKING | DTC: Pattern Recognition – Tính nhất quán giữa State Diagram và các model khác</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"State diagram của News/Post object có event DisableNews, EnableNews. Các event này có cần trùng tên với message trong sequence diagram và use case không? Hay đặt tên tự do cũng được?"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI RESPONSE (Summary): AI nói "Tên event trong state diagram đặt tự do miễn dễ hiểu, không nhất thiết trùng với sequence diagram vì chúng là các diagram độc lập."
-HUMAN DELTA &amp; REFLECTION:
-• Critical Thinking [Context Misunderstanding]: AI hiểu sai. Theo nguyên tắc mô hình hóa nhất quán (và như case study FOS minh họa rõ): các event gây chuyển trạng thái trong state diagram NÊN trùng tên với các message tương ứng đến state-dependent object trong sequence/communication diagram. Đây không phải bắt buộc cú pháp nhưng là best practice để đảm bảo traceability giữa các model.
-• Contextualization: Case study FOS (tài liệu RDS môn học) ghi rõ: "The events DisableNews and EnableNews cause state transitions to share the same names as two messages arriving at the state-dependent object in the sequence diagrams". Đây là chuẩn mực mà giảng viên dạy theo — AI không biết bối cảnh tài liệu môn học này.
-• Creative Synthesis: Tôi quyết định đồng bộ tên event xuyên suốt 3 model: trong sequence diagram có message DisableNews() gửi đến News object → trong state diagram News có transition Enable --&gt; Disable : DisableNews → trong use case có UC Disable News. Ba cái dùng chung 1 tên, tạo traceability.
-• Decision Ownership: Quyết định đặt tên event state diagram TRÙNG với message sequence diagram và tên use case. Lý do: đảm bảo tính nhất quán giữa các model (yêu cầu quan trọng khi chấm điểm), giúp người đọc và giảng viên truy vết từ use case → sequence → state. Không đặt tên tùy tiện như AI gợi ý.
-EVIDENCE: State diagram News/Post; sequence diagram Disable/Enable News; case study FOS (RDS) về tính nhất quán event-message.</t>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Pattern Recognition – Nhận diện Design Pattern đã dùng trong code IELTSPhobic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi có code IELTSPhobic với cấu trúc: mỗi entity có IRepository interface, Repository class implement interface, Service class inject repository qua constructor. Trong Design Patterns (GoF), pattern nào được áp dụng ở đây? Giải thích rõ từng pattern và tại sao nó phù hợp."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nhận ra Repository Pattern và Dependency Injection. AI nói "Repository Pattern là một GoF pattern thuộc nhóm Creational, tương tự Factory Pattern vì đều tạo object". AI giải thích DI là một behavioral pattern.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Fabrication]: AI SAI ở phân loại. Repository Pattern KHÔNG phải GoF pattern — nó là Architectural/Enterprise pattern (từ sách "Patterns of Enterprise Application Architecture" của Martin Fowler), không nằm trong 23 pattern GoF. Còn Dependency Injection cũng không phải GoF pattern — nó là application của Inversion of Control principle. AI trộn lẫn các nguồn khác nhau.
+• Contextualization: Pattern GoF thật sự trong code IELTSPhobic: (1) STRATEGY pattern — IWritingService, IExamService là interface, WritingService/ExamService là concrete strategy, controller chọn implementation qua DI; (2) FACADE pattern — mỗi Service class là facade che đi sự phức tạp của Repository + DbContext; (3) SINGLETON — ApplicationDbContext được đăng ký Scoped (1 instance/request) trong Program.cs.
+• Creative Synthesis: Tôi phân tách rõ: Repository Pattern = architectural pattern (không phải GoF); các GoF pattern thực sự dùng là Strategy (service interface), Facade (service layer), và Singleton-like (DbContext scoped). Ghi rõ pattern nào là GoF, pattern nào là architectural để tránh nhầm lẫn.
+• Decision Ownership: Quyết định chỉ tuyên bố GoF pattern khi chắc chắn đúng nguồn (sách Gamma 1995), không gộp các pattern từ nguồn khác vào. Lý do: PT1 và giảng viên hỏi về GoF — nếu nói sai nguồn sẽ mất điểm. Trích đúng: Strategy (behavioral), Facade (structural), Singleton (creational).
+EVIDENCE: Program.cs (Scoped DbContext = Singleton-like); IWritingService interface (Strategy); WritingService as Facade; sách Gamma 1995 (23 GoF patterns).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Pattern Recognition – Singleton Pattern: định nghĩa và áp dụng đúng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Singleton Pattern đảm bảo chỉ có 1 instance của class trong toàn bộ ứng dụng. Trong IELTSPhobic, ApplicationDbContext được đăng ký là Scoped (1 instance per HTTP request). Như vậy ApplicationDbContext có phải là Singleton Pattern không? OpenAIService đăng ký Singleton thì sao?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "DbContext Scoped và Singleton Pattern là giống nhau, vì cả hai đều đảm bảo chỉ có 1 instance. Scoped chỉ là một biến thể của Singleton trong ASP.NET Core." AI kết luận "dùng DbContext Scoped = đang áp dụng Singleton Pattern".
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Logic Error/Oversimplification]: AI SAI. Singleton Pattern (GoF) đảm bảo 1 instance DUY NHẤT trong TOÀN BỘ vòng đời ứng dụng (application lifetime). Còn Scoped = 1 instance per HTTP request — mỗi request tạo instance MỚI. Đây là 2 khái niệm khác nhau hoàn toàn. Nếu DbContext là Singleton thật (1 instance toàn app) thì sẽ xảy ra lỗi concurrency nghiêm trọng khi nhiều request dùng chung 1 DbContext.
+• Contextualization: Trong code IELTSPhobic, Program.cs đăng ký: DbContext = Scoped (đúng cho EF Core, mỗi request độc lập), OpenAIService = Singleton (đúng vì không có state, share được). Chỉ OpenAIService mới đúng Singleton Pattern GoF. Nhầm Scoped thành Singleton có thể dẫn đến bug nghiêm trọng nếu ai đó thay đổi registration.
+• Creative Synthesis: Tôi phân biệt rõ 3 lifetime trong ASP.NET Core: Singleton (1 instance/app lifetime = đúng GoF Singleton) → dùng cho stateless service như OpenAIService; Scoped (1/request) → DbContext; Transient (mỗi lần inject = new instance) → service nhẹ. Chỉ Singleton lifetime mới tương đương GoF Singleton Pattern.
+• Decision Ownership: Quyết định chỉ công nhận OpenAIService là Singleton Pattern (GoF), DbContext Scoped KHÔNG phải Singleton. Lý do: đúng định nghĩa GoF (application lifetime) và tránh nhầm lẫn gây bug khi maintain code sau này.
+CORRECTIVE ACTION: Sửa tuyên bố: Singleton GoF = OpenAIService (Singleton lifetime); DbContext Scoped ≠ Singleton Pattern.
+EVIDENCE: Program.cs (Scoped vs Singleton registration); GoF Singleton định nghĩa (1 instance/application lifetime); EF Core docs (DbContext phải Scoped).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Pattern Recognition – Strategy Pattern: nhận diện và vẽ class diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"IELTSPhobic có IOpenAIService interface và OpenAIService implementation. Trong tương lai có thể thêm GeminiService hoặc ClaudeService để thay thế. Pattern nào phù hợp để mô hình hóa việc này? Vẽ class diagram minh họa."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nhận ra đây là Strategy Pattern (behavioral): định nghĩa một family of algorithms, encapsulate từng cái, cho phép thay đổi lẫn nhau. AI đề xuất: AIContext (context) giữ reference đến IAIService (strategy interface), OpenAIService/GeminiService/ClaudeService là concrete strategies.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG — đây đúng là Strategy Pattern. Tôi kiểm chứng với GoF: Strategy = interface + nhiều implementation hoán đổi được, client dùng qua interface mà không biết concrete class. Cấu trúc khớp: IOpenAIService (Strategy interface), OpenAIService (Concrete Strategy), WritingService (Context dùng strategy qua DI).
+• Contextualization: AI đề xuất thêm class "AIContext" riêng, nhưng trong code thực tế không cần class Context riêng vì ASP.NET Core DI đóng vai trò Context — inject đúng implementation tùy cấu hình. Đây là điểm tinh tế mà AI không biết vì không đọc code.
+• Creative Synthesis: Tôi vẽ class diagram Strategy Pattern gọn hơn: IOpenAIService (interface, strategy) với các method AnalyzeWriting() + AnalyzeSpeaking(); OpenAIService implements IOpenAIService; WritingService (context) có field _aiService: IOpenAIService inject qua constructor. Không cần AIContext riêng. Thêm ghi chú "future: GeminiService, ClaudeService có thể thay thế không cần sửa WritingService".
+• Decision Ownership: Quyết định vẽ Strategy Pattern bỏ class Context riêng, dùng DI làm context thay thế. Lý do: khớp code thật, không vẽ thêm abstraction không cần thiết. Thể hiện Strategy Pattern "thực chiến" trong ASP.NET Core, không chỉ theo sách lý thuyết.
+EVIDENCE: IOpenAIService.cs, OpenAIService.cs, WritingService.cs trong repo; GoF Strategy Pattern (behavioral); class diagram minh họa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICATION | DTC: Abstraction – Observer Pattern vs Event-driven: phân biệt đúng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong IELTSPhobic, khi exam attempt được submit, hệ thống tự động trigger AI feedback cho Writing/Speaking. Khi user mua VIP, hệ thống gửi email xác nhận. Những luồng này có phải Observer Pattern không? Observer Pattern là gì?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI trả lời "Đúng, cả hai luồng đều là Observer Pattern. Observer Pattern là khi một object (Subject) thay đổi trạng thái thì tự động notify tất cả observers. Exam attempt submit = Subject notify AI service; VIP payment = Subject notify Email service. Đây là Observer Pattern chuẩn GoF."
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [HALLUCINATION – Context Misunderstanding]: AI áp dụng sai. Observer Pattern (GoF) yêu cầu: Subject giữ danh sách Observer, chủ động gọi Notify() khi state thay đổi, Observer register/unregister vào Subject. Trong code IELTSPhobic, không có cơ chế register/unregister observer — khi submit exam, WritingService chỉ gọi thẳng OpenAIService.AnalyzeWriting() (synchronous call, không qua observer list). Khi VIP, StripeWebhookService gọi thẳng EmailService. Đây là DIRECT CALL, không phải Observer Pattern.
+• Contextualization: Để thật sự dùng Observer Pattern, code cần: IObserver interface với method Update(), Subject có List&lt;IObserver&gt; và Notify() loop. Hiện tại code dùng cách đơn giản hơn (direct dependency injection). AI nhầm vì thấy "một việc trigger việc khác" liền nghĩ Observer, nhưng trigger ≠ Observer Pattern.
+• Creative Synthesis: Tôi phân biệt: luồng hiện tại là DIRECT CALL (Service A gọi thẳng Service B qua DI). Nếu muốn dùng Observer Pattern thật, cần thêm: IAttemptObserver interface, ExamAttemptService register observer list, AIFeedback Observer + NotificationObserver implement interface. Đây là cải tiến có thể làm cho kiến trúc linh hoạt hơn (thêm observer mà không sửa ExamAttemptService).
+• Decision Ownership: Quyết định KHÔNG tuyên bố code hiện tại dùng Observer Pattern. Ghi nhận đây là Direct Call, đề xuất refactor sang Observer nếu cần mở rộng. Lý do: khai báo pattern không đúng sẽ bị giảng viên bắt bẻ khi vấn đáp đối chiếu code.
+CORRECTIVE ACTION: Không gán Observer cho luồng submit/VIP hiện tại; ghi là "Direct call, potential Observer refactor".
+EVIDENCE: WritingService.cs (direct call OpenAIService); GoF Observer định nghĩa (Subject + Observer list + Notify loop).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING | DTC: Pattern Recognition – Facade Pattern: đơn giản hóa giao diện phức tạp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"ExamService trong IELTSPhobic phải phối hợp: ExamRepository (lấy data), CloudinaryService (upload audio), OpenAIService (AI scoring), EmailService (gửi mail). Controller chỉ gọi ExamService mà không biết các dependency bên trong. Pattern nào đây và ưu điểm là gì?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nhận ra đây là Facade Pattern (structural): ExamService là Facade đứng trước một tập hợp các subsystem phức tạp, cung cấp interface đơn giản cho ExamController. AI giải thích ưu điểm: giảm coupling, Controller không cần biết chi tiết Cloudinary/OpenAI/Email.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking: AI ĐÚNG — Facade Pattern (GoF, Structural) phù hợp. Tôi kiểm chứng với định nghĩa GoF: Facade cung cấp unified interface đơn giản hơn cho một tập subsystem, giảm dependency của client vào subsystem. ExamService làm đúng điều này: ExamController chỉ cần biết IExamService với vài method, không biết gì về Cloudinary, OpenAI hay Email bên dưới.
+• Contextualization: AI chưa đề cập một ưu điểm quan trọng trong bối cảnh project: Facade + Interface (IExamService) giúp testability — có thể mock IExamService trong unit test mà không cần real Cloudinary/OpenAI. Đây là lý do thực tế tôi chọn pattern này, không chỉ để "đẹp".
+• Creative Synthesis: Tôi xác nhận ExamService = Facade Pattern và bổ sung vào class diagram: ExamController chỉ thấy IExamService (simplified interface); bên trong ExamService phối hợp IExamRepository + ICloudinaryService + IOpenAIService + EmailService (subsystems). Thêm ghi chú ưu điểm: loose coupling + testability + dễ thay Cloudinary bằng AWS S3 mà không đụng Controller.
+• Decision Ownership: Quyết định công nhận Facade Pattern và document rõ trong báo cáo kèm class diagram. Lý do: đây là GoF pattern thật sự có trong code, có thể giải thích được khi vấn đáp, và là điểm mạnh kỹ thuật của kiến trúc nhóm so với các nhóm chỉ viết code không theo pattern.
+EVIDENCE: ExamService.cs (Facade); ExamController.cs (chỉ gọi IExamService); GoF Facade Pattern (structural); class diagram Facade IELTSPhobic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION-MAKING | DTC: Abstraction – Document Design Pattern đúng chuẩn GoF trong báo cáo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Khi báo cáo SWD392 yêu cầu "explain the structure and document a Design Pattern" (CLO6), tôi nên document pattern theo format nào? Cần bao nhiêu pattern và mức độ chi tiết thế nào?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI RESPONSE (Summary): AI nói "document pattern bằng cách copy định nghĩa từ internet, liệt kê 10+ pattern đang dùng trong code để thể hiện phong phú". AI gợi ý format: tên pattern + 1 câu mô tả + code snippet.
+HUMAN DELTA &amp; REFLECTION:
+• Critical Thinking [Oversimplification]: AI sai cả về format lẫn số lượng. Theo syllabus CLO6 "explain the structure and document a Design Pattern" và tài liệu GoF, document một pattern chuẩn phải gồm: Name, Problem (bối cảnh vấn đề), Solution (cấu trúc class diagram + mô tả), Consequences (ưu/nhược điểm, trade-off). Copy định nghĩa internet không phải "document" — phải áp dụng vào hệ thống thật. Liệt kê 10+ pattern sơ sài hơn 3 pattern chi tiết.
+• Contextualization: Trong bối cảnh báo cáo nhóm, session 22 (PT1 + On-going Assessment 1) yêu cầu giảng viên có thể hỏi vấn đáp về pattern. Nếu chỉ copy tên pattern mà không giải thích được problem/solution/consequences trong ngữ cảnh IELTSPhobic, sẽ không đạt.
+• Creative Synthesis: Tôi chọn document 3 pattern thật sự có trong code (Strategy, Facade, Singleton), mỗi cái theo format đầy đủ GoF: (1) Name, (2) Problem — vấn đề gì trong IELTSPhobic cần giải quyết, (3) Solution — class diagram + giải thích các vai trò, (4) Consequences — ưu điểm (loose coupling, extensible) và nhược điểm (thêm abstraction layer). Gắn code snippet thật từ repo vào phần Solution.
+• Decision Ownership: Quyết định document 3 pattern theo đúng format GoF 4 mục, KHÔNG liệt kê nhiều pattern sơ sài. Lý do: chất lượng hơn số lượng — 3 pattern hiểu sâu + giải thích được context IELTSPhobic sẽ đạt CLO6 tốt hơn 10 pattern copy-paste. Đây cũng là chuẩn mà giảng viên hỏi vấn đáp.
+EVIDENCE: Báo cáo Section V.Design Patterns với 3 pattern (Strategy/Facade/Singleton) theo format GoF 4 mục; syllabus CLO6; sách Gamma 1995 (pattern template).</t>
   </si>
 </sst>
 </file>
@@ -1480,107 +1573,107 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="69.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="71.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="n">
+    <row r="2" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="16" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="n">
+      <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="16" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="344.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="n">
+    <row r="4" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="16" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="449.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="n">
+    <row r="5" customFormat="false" ht="464.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="16" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="n">
+    <row r="6" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="16" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="344.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="n">
+    <row r="7" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="16" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1606,7 +1699,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="71.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="69.8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1623,7 +1716,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
@@ -1637,7 +1730,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="404.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="419.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
@@ -1651,7 +1744,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="n">
         <v>3</v>
       </c>
@@ -1665,7 +1758,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="464.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="449.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
@@ -1693,7 +1786,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
@@ -1705,6 +1798,129 @@
       </c>
       <c r="D7" s="16" t="s">
         <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="82"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="389.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="434.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="374.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>